<commit_message>
Update state - 2026-07-26
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="mmmm d, yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mmmm d, yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,12 +49,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -133,7 +133,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K17" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K19" headerRowCount="1">
   <autoFilter ref="A1:K17"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -472,7 +472,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
@@ -548,7 +548,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="3" t="n">
         <v>46279</v>
       </c>
       <c r="E2" t="inlineStr">
@@ -601,7 +601,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="3" t="n">
         <v>46496</v>
       </c>
       <c r="E3" t="inlineStr">
@@ -654,7 +654,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="3" t="n">
         <v>46678</v>
       </c>
       <c r="E4" t="inlineStr">
@@ -707,7 +707,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="3" t="n">
         <v>46231</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -720,7 +720,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/mwFE8ZYhmC3Ce</t>
@@ -756,7 +755,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="3" t="n">
         <v>46233</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -769,7 +768,6 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/ibm-skillsbuild-orientation-1693369?sourceTypeId=Website</t>
@@ -805,7 +803,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="3" t="n">
         <v>46239</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -818,7 +816,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/MwFNl0es8CeCg</t>
@@ -850,7 +847,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="3" t="n">
         <v>46240</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -863,7 +860,6 @@
           <t>4:00 PM - 12:30 PM</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/rural-ai-workforce-forum-2026-1759715?sourceTypeId=Website</t>
@@ -899,7 +895,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="3" t="n">
         <v>46247</v>
       </c>
       <c r="E9" t="inlineStr">
@@ -912,7 +908,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/WqFgM07iaCJCE</t>
@@ -948,7 +943,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="3" t="n">
         <v>46252</v>
       </c>
       <c r="E10" t="inlineStr">
@@ -961,7 +956,6 @@
           <t>8:00 AM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/12F2XblUgCVCB</t>
@@ -993,7 +987,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="3" t="n">
         <v>46261</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -1006,7 +1000,6 @@
           <t>5:00 PM - 7:45 PM</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/xRF50ZqHMCYC7</t>
@@ -1042,7 +1035,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="3" t="n">
         <v>46261</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -1055,7 +1048,6 @@
           <t>6:00 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/EqFedRnCgC6C9</t>
@@ -1091,7 +1083,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="3" t="n">
         <v>46280</v>
       </c>
       <c r="E13" t="inlineStr">
@@ -1104,7 +1096,6 @@
           <t>10:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/OOFNE8dhaCqCD</t>
@@ -1136,7 +1127,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="3" t="n">
         <v>46282</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -1149,7 +1140,6 @@
           <t>5:30 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/beyond-connected-iot-s-next-chapter-presented-by-tag-cloud-society-1848946?sourceTypeId=Website</t>
@@ -1185,7 +1175,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="3" t="n">
         <v>46283</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -1198,7 +1188,6 @@
           <t>8:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/R1Fo7y2FRC0CX</t>
@@ -1234,7 +1223,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="3" t="n">
         <v>46303</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -1247,7 +1236,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/kgFYW1VuzCVC1</t>
@@ -1283,7 +1271,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D17" s="3" t="n">
         <v>46317</v>
       </c>
       <c r="E17" t="inlineStr">
@@ -1296,7 +1284,6 @@
           <t>1:00 PM - 5:00 PM</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/QZFMBR6tdCnC0</t>
@@ -1317,6 +1304,56 @@
           <t>While TAG is a Georgia-focused organization and this is a pitch/networking event for tech entrepreneurs, the event description has zero mention of AI, machine learning, or automation, making it an automatic low score; the virtual-only format with a Georgia org prevents it from being a 1, but the lack of AI content keeps it at 2.</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/events</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>July 26, 2026</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>failed: unexpected error: Connection error.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>July 26, 2026</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>failed: unexpected error: Connection error.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1419,7 +1456,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="3" t="n">
         <v>46232</v>
       </c>
       <c r="E2" t="inlineStr">
@@ -1432,7 +1469,6 @@
           <t>5:00 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/israeli-cybersecurity-summit-1360489?sourceTypeId=Website</t>
@@ -1464,7 +1500,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="3" t="n">
         <v>46237</v>
       </c>
       <c r="E3" t="inlineStr">
@@ -1477,7 +1513,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/EqF6GN4IgC6C9</t>
@@ -1513,7 +1548,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="3" t="n">
         <v>46238</v>
       </c>
       <c r="E4" t="inlineStr">
@@ -1526,7 +1561,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/VeFAOextNCeC9</t>
@@ -1562,7 +1596,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="3" t="n">
         <v>46246</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -1575,7 +1609,6 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/qWFX016fkCQCe</t>
@@ -1611,7 +1644,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="3" t="n">
         <v>46266</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -1624,7 +1657,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/7EFZQMQsNCQCd</t>
@@ -1656,7 +1688,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="3" t="n">
         <v>46279</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -1669,7 +1701,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/VeFXK8WSNCeC9</t>
@@ -1705,7 +1736,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="3" t="n">
         <v>46300</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -1718,7 +1749,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/nvF6MwdSECNCZ</t>
@@ -1754,7 +1784,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="3" t="n">
         <v>46301</v>
       </c>
       <c r="E9" t="inlineStr">
@@ -1767,7 +1797,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/3BFg2ejHYCQCg</t>
@@ -1799,7 +1828,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="3" t="n">
         <v>46328</v>
       </c>
       <c r="E10" t="inlineStr">
@@ -1812,7 +1841,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/jKFGO1mfZCkCE</t>
@@ -1848,7 +1876,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="3" t="n">
         <v>46329</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -1861,7 +1889,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/9eFlWx1fWC9Cx</t>
@@ -1893,7 +1920,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="3" t="n">
         <v>46331</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -1906,7 +1933,6 @@
           <t>11:30 AM - 2:00 PM</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/pending-veterans-day-presented-by-tag-infrastructure-society-1775943?sourceTypeId=Website</t>
@@ -1938,7 +1964,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="3" t="n">
         <v>46345</v>
       </c>
       <c r="E13" t="inlineStr">
@@ -1951,7 +1977,6 @@
           <t>6:00 PM - 11:00 PM</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/tag-chairs-gala-2026-1569285?sourceTypeId=Website</t>
@@ -1983,7 +2008,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="3" t="n">
         <v>46357</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -1996,7 +2021,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/xRFXAz4IMCYC7</t>
@@ -2028,7 +2052,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="3" t="n">
         <v>46360</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -2041,7 +2065,6 @@
           <t>9:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/oXFq4V1T6C2CB</t>
@@ -2077,7 +2100,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="3" t="n">
         <v>46363</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -2090,7 +2113,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/G9FwqlWUNCxCK</t>

</xml_diff>

<commit_message>
Update state - 2026-07-27
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="mmmm d, yyyy"/>
+    <numFmt numFmtId="164" formatCode="mmmm d, yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -50,12 +50,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -133,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K53" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K83" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -153,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K132" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K153" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -461,18 +462,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
@@ -548,7 +549,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="3" t="n">
         <v>46252</v>
       </c>
       <c r="E2" t="inlineStr">
@@ -556,7 +557,6 @@
           <t>July 2, 2026</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Renaissance Atlanta Waverly Hotel &amp; Convention Center, 2450 Galleria Pkwy, Atlanta, GA 30339</t>
@@ -597,7 +597,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="3" t="n">
         <v>46249</v>
       </c>
       <c r="E3" t="inlineStr">
@@ -650,7 +650,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="3" t="n">
         <v>46678</v>
       </c>
       <c r="E4" t="inlineStr">
@@ -703,7 +703,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="3" t="n">
         <v>46234</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -752,7 +752,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="3" t="n">
         <v>46225</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -801,7 +801,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="3" t="n">
         <v>46215</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -850,7 +850,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -899,7 +899,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="3" t="n">
         <v>46218</v>
       </c>
       <c r="E9" t="inlineStr">
@@ -948,7 +948,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="3" t="n">
         <v>46206</v>
       </c>
       <c r="E10" t="inlineStr">
@@ -997,7 +997,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="3" t="n">
         <v>46233</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -1046,7 +1046,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="3" t="n">
         <v>46239</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -1099,7 +1099,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="3" t="n">
         <v>46267</v>
       </c>
       <c r="E13" t="inlineStr">
@@ -1152,7 +1152,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="3" t="n">
         <v>46302</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -1205,7 +1205,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -1218,7 +1218,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -1254,7 +1253,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="3" t="n">
         <v>46238</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -1267,7 +1266,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -1303,7 +1301,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D17" s="3" t="n">
         <v>46280</v>
       </c>
       <c r="E17" t="inlineStr">
@@ -1316,7 +1314,6 @@
           <t>10:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -1348,7 +1345,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="3" t="n">
         <v>46216</v>
       </c>
       <c r="E18" t="inlineStr">
@@ -1397,7 +1394,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D19" s="1" t="n">
+      <c r="D19" s="3" t="n">
         <v>46279</v>
       </c>
       <c r="E19" t="inlineStr">
@@ -1450,7 +1447,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="D20" s="3" t="n">
         <v>46496</v>
       </c>
       <c r="E20" t="inlineStr">
@@ -1503,7 +1500,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>August 18, 2026 - August 20, 2026</t>
         </is>
@@ -1513,8 +1510,6 @@
           <t>July 2, 2026</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/ *</t>
@@ -1546,7 +1541,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>August 6-7, 2026</t>
         </is>
@@ -1561,7 +1556,6 @@
           <t>4:00 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -1597,7 +1591,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D23" s="1" t="n">
+      <c r="D23" s="3" t="n">
         <v>46283</v>
       </c>
       <c r="E23" t="inlineStr">
@@ -1610,7 +1604,6 @@
           <t>8:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -1646,7 +1639,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D24" s="1" t="n">
+      <c r="D24" s="3" t="n">
         <v>46303</v>
       </c>
       <c r="E24" t="inlineStr">
@@ -1699,7 +1692,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D25" s="1" t="n">
+      <c r="D25" s="3" t="n">
         <v>46360</v>
       </c>
       <c r="E25" t="inlineStr">
@@ -1712,7 +1705,6 @@
           <t>9:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -1748,7 +1740,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D26" s="1" t="n">
+      <c r="D26" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="E26" t="inlineStr">
@@ -1797,7 +1789,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D27" s="1" t="n">
+      <c r="D27" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E27" t="inlineStr">
@@ -1846,7 +1838,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="D28" s="3" t="n">
         <v>46205</v>
       </c>
       <c r="E28" t="inlineStr">
@@ -1895,7 +1887,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D29" s="1" t="n">
+      <c r="D29" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E29" t="inlineStr">
@@ -1944,7 +1936,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D30" s="1" t="n">
+      <c r="D30" s="3" t="n">
         <v>46223</v>
       </c>
       <c r="E30" t="inlineStr">
@@ -1993,7 +1985,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D31" s="1" t="n">
+      <c r="D31" s="3" t="n">
         <v>46224</v>
       </c>
       <c r="E31" t="inlineStr">
@@ -2042,7 +2034,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D32" s="1" t="n">
+      <c r="D32" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E32" t="inlineStr">
@@ -2091,7 +2083,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="3" t="n">
         <v>46220</v>
       </c>
       <c r="E33" t="inlineStr">
@@ -2140,7 +2132,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D34" s="1" t="n">
+      <c r="D34" s="3" t="n">
         <v>46217</v>
       </c>
       <c r="E34" t="inlineStr">
@@ -2193,7 +2185,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D35" s="1" t="n">
+      <c r="D35" s="3" t="n">
         <v>46232</v>
       </c>
       <c r="E35" t="inlineStr">
@@ -2206,7 +2198,6 @@
           <t>5:00 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -2238,7 +2229,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D36" s="1" t="n">
+      <c r="D36" s="3" t="n">
         <v>46252</v>
       </c>
       <c r="E36" t="inlineStr">
@@ -2251,7 +2242,6 @@
           <t>8:00 AM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -2283,7 +2273,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D37" s="1" t="n">
+      <c r="D37" s="3" t="n">
         <v>46301</v>
       </c>
       <c r="E37" t="inlineStr">
@@ -2296,7 +2286,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -2328,7 +2317,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D38" s="1" t="n">
+      <c r="D38" s="3" t="n">
         <v>46331</v>
       </c>
       <c r="E38" t="inlineStr">
@@ -2341,7 +2330,6 @@
           <t>11:30 AM - 2:00 PM</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -2373,7 +2361,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D39" s="1" t="n">
+      <c r="D39" s="3" t="n">
         <v>46345</v>
       </c>
       <c r="E39" t="inlineStr">
@@ -2386,7 +2374,6 @@
           <t>6:00 PM - 11:00 PM</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -2418,7 +2405,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D40" s="1" t="n">
+      <c r="D40" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="E40" t="inlineStr">
@@ -2467,7 +2454,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D41" s="1" t="n">
+      <c r="D41" s="3" t="n">
         <v>46227</v>
       </c>
       <c r="E41" t="inlineStr">
@@ -2516,7 +2503,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D42" s="1" t="n">
+      <c r="D42" s="3" t="n">
         <v>46205</v>
       </c>
       <c r="E42" t="inlineStr">
@@ -2565,7 +2552,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D43" s="1" t="n">
+      <c r="D43" s="3" t="n">
         <v>46205</v>
       </c>
       <c r="E43" t="inlineStr">
@@ -2614,7 +2601,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D44" s="1" t="n">
+      <c r="D44" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E44" t="inlineStr">
@@ -2663,7 +2650,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D45" s="1" t="n">
+      <c r="D45" s="3" t="n">
         <v>46205</v>
       </c>
       <c r="E45" t="inlineStr">
@@ -2712,7 +2699,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D46" s="1" t="n">
+      <c r="D46" s="3" t="n">
         <v>46215</v>
       </c>
       <c r="E46" t="inlineStr">
@@ -2761,7 +2748,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D47" s="1" t="n">
+      <c r="D47" s="3" t="n">
         <v>46205</v>
       </c>
       <c r="E47" t="inlineStr">
@@ -2810,7 +2797,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D48" s="1" t="n">
+      <c r="D48" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E48" t="inlineStr">
@@ -2823,7 +2810,6 @@
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>https://luma.com/genai-collective *</t>
@@ -2855,7 +2841,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D49" s="1" t="n">
+      <c r="D49" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E49" t="inlineStr">
@@ -2904,7 +2890,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D50" s="1" t="n">
+      <c r="D50" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="E50" t="inlineStr">
@@ -2953,7 +2939,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D51" s="1" t="n">
+      <c r="D51" s="3" t="n">
         <v>46225</v>
       </c>
       <c r="E51" t="inlineStr">
@@ -3002,7 +2988,7 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D52" s="1" t="n">
+      <c r="D52" s="3" t="n">
         <v>46239</v>
       </c>
       <c r="E52" t="inlineStr">
@@ -3051,7 +3037,7 @@
           <t>medium</t>
         </is>
       </c>
-      <c r="D53" s="1" t="n">
+      <c r="D53" s="3" t="n">
         <v>46205</v>
       </c>
       <c r="E53" t="inlineStr">
@@ -3085,6 +3071,1390 @@
           <t>While the event is in-person in Atlanta, there is zero mention of AI, machine learning, or automation, which is an automatic disqualifier regardless of location.</t>
         </is>
       </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Tech AI Symposium and AI Career Fair</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>5</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>9:45 AM EDT</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Exhibition Hall (460 4th St NW, Atlanta, GA 30332)</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/tech-ai-symposium-and-ai-career-fair</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech's premier event connecting students, researchers, faculty, industry leaders, and employers to explore the future of artificial intelligence.</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>In-person Georgia Tech AI event in Atlanta with clear AI focus, career fair component, and confirmed September 2026 date at a specific Georgia location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Cyber Resilience in the AI Era presented by TAG Cybersecurity &amp; Risk Management Society and TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/MwFNl0es8CeCg</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Virtual event with clear AI content (presented by TAG Data Science &amp; AI Society) and cybersecurity focus, hosted by a Georgia-focused organization (TAG), scoring well despite virtual format and missing description details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Rural AI Workforce Forum 2026</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>4:00 PM - 12:30 PM</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/rural-ai-workforce-forum-2026-1759715?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Preparing rural communities for an AI-driven future.</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Virtual event with clear AI content hosted by TAG (a Georgia-based organization), but lacks specific details about format, speakers, and actual Georgia focus beyond the organizer's location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>From Forecasting to Demand Orchestration: How AI Is Redefining Supply Chain Planning presented by TAG Data Science &amp; AI Society and TAG Supply Chain, Logistics &amp; Manufacturing Society</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/WqFgM07iaCJCE</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>You'll hear what's working now, what's still hard, and how companies across utilities, healthcare, financial services, retail, and CPG are using AI to move faster and smarter.</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Virtual event with strong AI content (demand orchestration, AI in supply chain planning) hosted by TAG (Atlanta-based organization), but lacks confirmed Georgia focus and location details lower the score from what an in-person version would achieve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>AI Superpowers for Good: Solving Society's Biggest Challenges presented by TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>5:00 PM - 7:45 PM</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/xRF50ZqHMCYC7</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>An inspiring evening showcasing complete, real-world data science and AI projects from concept to impact.</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Virtual event with clear AI content hosted by TAG (a Georgia-focused organization), but lacks specific location confirmation and detailed description that would elevate it higher.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>IBM Certificate (in-Person) Graduation</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/EqFedRnCgC6C9</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a special virtual celebration honoring the achievements of participants in the IBM SkillsBuild Program. This event recognizes learners from our recent cohorts who have dedicated their time and effort to building in-demand skills.</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>Event has AI/tech content (IBM SkillsBuild) and is hosted by TAG (Georgia-focused org), but is a graduation ceremony celebrating past learning rather than an educational AI event itself, and location field is blank despite in-person claim creating ambiguity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Beyond Connected: IoT's Next Chapter presented by TAG Cloud Society</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>5:30 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/beyond-connected-iot-s-next-chapter-presented-by-tag-cloud-society-1848946?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>An executive panel exploring how leading organizations are transforming connected devices into intelligent, business-driven ecosystems.</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Virtual event hosted by TAG (Georgia-based organization) with AI/automation relevance through IoT and intelligent systems discussion, scoring 3-4 range for Georgia institution virtual content, but lacks explicit AI/ML terminology and location ambiguity slightly reduces confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Manufacturing Technology Challenges: Practical Solutions for Today's Pla...</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>11:00 AM - 1:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/tech-educational-panel</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>The event description is empty and the title gives no indication of AI, machine learning, or automation content, making it impossible to confirm AI relevance despite the Georgia-focused organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>AIMST 2026 Atlanta</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Renaissance Atlanta Waverly Hotel &amp; Convention Center, 2450 Galleria Pkwy, Atlanta, GA 30339</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.meetmax.com/sched/event_130973/conference_register.html?attendee_role_id=TWST2_ATTENDEE&amp;grp_name=ATTENDEE&amp;approved=Y&amp;_gl=1*g58gv2*_gcl_au*Mjc2MTM5ODY0LjE3ODEwMTU3MjQ.*_ga*MTYwNTkxMjEyNC4xNzU2MjA4NDM5*_ga_M7N3QCZSH0*czE3ODM5OTUzOTAkbzExNCRnMSR0MTc4Mzk5NjQ2NiRqMzkkbDAkaDA.</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>North America's #1 Conference in Industrial AI, focused on providing in-depth discussions and solutions for heads of manufacturing, advanced technology managers, ICS, IT/OT, SCADA and cyber security professionals to accelerate their digital transformation and transform their operational and automation systems. Features three tech tracks (AI Manufacturing, Industrial AI 101 for SMEs, SCADA Technology &amp; AI Utilities), 60+ speakers, 350+ attendees, and 8+ networking events.</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>AIMST 2026 is an in-person industrial AI conference in Atlanta with substantial AI content (three AI-focused tech tracks, 60+ speakers, 350+ attendees), meeting all criteria for excellent fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>TechConnect: Global Virtual Job &amp; Networking Event for Data, AI, and Tech Pros</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>4:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ac-atl/events/313188287/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-online&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only national job fair with AI content mentions, but lacks Georgia-specific focus and has no detailed description to confirm educational value versus recruitment pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Atlanta Tech Meet-Up</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46238</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atl-tech-meetup/events/315779247/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>FREE REMOTE | LADIES IN AI - We Learn. We Share. We Laugh.</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/315016411/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-online&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with AI content (Ladies in AI community group) but no Georgia-specific focus and lacks detailed description to assess educational value beyond community gathering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Agentic AI Meetup - August</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>4</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>5:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/aittg-atlanta/events/315755582/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI meetup (Agentic AI) hosted by Atlanta-based AITTG organization with strong AI content focus, but confidence is medium due to missing location details and empty description field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Bytes &amp; Bites: Atlanta Tech Week Edition @ Krog St Market</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>11:45 AM EDT</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Krog St Market</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/315763802/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Atlanta location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Building an AI resume optimization tool with Matthew Christiansen: Session 2</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/google-developer-groups-gdg-atlanta/events/315294142/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-online&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Virtual event with AI/ML content (resume optimization tool) hosted by GDG Atlanta (Georgia-focused organization) scores above typical national corporate webinars, but lacks in-person presence and detailed description limits full assessment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>AWS + HashiCorp Terraform DevOps GameDay</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlanta-aws-user-group/events/315805518/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Event lacks AI/ML/automation content in title and description (automatic 1 territory), but is in-person with Atlanta AWS user group affiliation which provides minimal uplift; however, the missing location field and empty description create significant ambiguity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" s="3" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Building Intelligent AI Agents with GraphRAG</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>9:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/building-intelligent-ai-agents-with-graphrag-tickets-1992756563525?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Event has clear AI content (GraphRAG and intelligent agents) but is virtual-only with no indication of Georgia focus or Georgia institution involvement, and lacks sufficient details to determine if it's educational or sales-focused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Those Time Drains and Money Leaks? AI Should Be Fixing That. Find Out How.</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/those-time-drains-and-money-leaks-ai-should-be-fixing-that-find-out-how-tickets-1995249007492?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Event has AI content in title but lacks description, location details, and Georgia focus; virtual-only format with vague sales-pitch-style title suggesting a promotional webinar rather than substantive educational content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Atlanta Tech Mixer and Social (Tech / AI / Data / IT) ✨</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Atlanta · Stats Brewpub</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/atlanta-tech-mixer-and-social-tech-ai-data-it-tickets-1987408339844?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>While this is an in-person Atlanta event with AI mentioned in the title, it appears to be a generic networking mixer rather than an educational AI event with substantive content, and the complete lack of description makes it difficult to assess the actual focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Data Science with Phython Certification Training in Columbus, GA</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>2</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Columbus · Veterans Parkway</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/data-science-with-phython-certification-training-in-columbus-ga-tickets-1984660920238?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>While the event is in-person in Georgia (Columbus), it appears to be a paid certification training focused on Python/data science rather than an educational event about AI/ML concepts, and the empty description makes it difficult to assess actual AI content relevance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Everything but the Camera: ACS</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Atlanta · Atlanta Axis Experience Center</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/everything-but-the-camera-acs-tickets-1990888109930?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, making it an automatic 1 regardless of location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Wednesd.AI</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>4</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Atlanta · Atlanta Tech Village - Buckhead</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>In-person event in Atlanta with AI-focused title (Wednesd.AI) suggesting regular AI content, but lack of detailed description creates some uncertainty about the specific content and educational value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>AI for the real World: Week 4: Make a Talking Video with AI (HeyGen Part 1</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>4</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>East Point · 1928 Stanton Rd</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-for-the-real-world-week-4-make-a-talking-video-with-ai-heygen-part-1-tickets-1992736032115?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI event in Georgia (East Point) with clear AI/automation content (video generation with HeyGen), though short description and part-of-series nature suggest it may be training-focused rather than purely educational.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tech, AI &amp; Startups Roundtable Discussion Dinner</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>4</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Atlanta · Aviva by Kameel Buckhead</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tech-ai-startups-roundtable-discussion-dinner-tickets-1988373794545?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>In-person event in Atlanta with explicit AI focus in the title, though the empty short description and roundtable dinner format (rather than technical content) prevent a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>AI Awareness: The Good, the Bad, and What to Watch For</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-awareness-the-good-the-bad-and-what-to-watch-for-tickets-1991930436557?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>Event clearly has AI content in its title, but is virtual-only with no Georgia focus mentioned, missing date/time/location details, and no description to assess whether it's educational or a sales pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Microsoft Copilot Cowork Masterclass</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46234</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>10:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/microsoft-copilot-cowork-masterclass-tickets-1990549050795?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>Event clearly mentions AI (Microsoft Copilot), but is virtual-only with no Georgia connection and appears to be a corporate training/sales pitch rather than educational content, and the empty short description limits confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>FREE Data Analytics with GenAI Bootcamp | USA Only |Join WhatsApp Group</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>10:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-data-analytics-with-genai-bootcamp-usa-only-join-whatsapp-group-tickets-1990886211251?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with clear AI/GenAI content but no Georgia focus, missing location details, and a bootcamp structure that suggests potential sales orientation rather than pure education.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>AI Tinkerers Atlanta: 2-Year Anniversary &amp; Best Demos of the Year</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>5</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>4:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/p/ai-tinkerers-atlanta-2-year-anniversary-best-demos-of-the-year</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>AI Tinkerers Atlanta will celebrate two years by showcasing impactful technical discoveries and working code. RenderATL Group will sponsor this community event.</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>In-person technical AI event in Atlanta celebrating community achievements with demos and code, combining Georgia location preference with strong AI content and educational value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3100,14 +4470,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -3187,7 +4557,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D2" s="1" t="n">
+      <c r="D2" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E2" t="inlineStr">
@@ -3236,7 +4606,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D3" s="1" t="n">
+      <c r="D3" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="E3" t="inlineStr">
@@ -3285,7 +4655,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="E4" t="inlineStr">
@@ -3334,7 +4704,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="3" t="n">
         <v>46225</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -3347,7 +4717,6 @@
           <t>11:00 AM - 1:00 PM EDT</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/ *</t>
@@ -3379,7 +4748,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="3" t="n">
         <v>46233</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -3428,7 +4797,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="3" t="n">
         <v>46233</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -3477,7 +4846,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="3" t="n">
         <v>46239</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -3490,7 +4859,6 @@
           <t>11:00 AM - 1:30 PM EDT</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/ *</t>
@@ -3522,7 +4890,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="3" t="n">
         <v>46245</v>
       </c>
       <c r="E9" t="inlineStr">
@@ -3535,7 +4903,6 @@
           <t>3:30 PM - 4:30 PM EDT</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/ *</t>
@@ -3567,7 +4934,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="3" t="n">
         <v>46254</v>
       </c>
       <c r="E10" t="inlineStr">
@@ -3616,7 +4983,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="3" t="n">
         <v>46254</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -3665,7 +5032,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="3" t="n">
         <v>46280</v>
       </c>
       <c r="E12" t="inlineStr">
@@ -3714,7 +5081,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="3" t="n">
         <v>46209</v>
       </c>
       <c r="E13" t="inlineStr">
@@ -3727,7 +5094,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -3763,7 +5129,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="E14" t="inlineStr">
@@ -3776,7 +5142,6 @@
           <t>3:00 PM - 6:30 PM</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -3812,7 +5177,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="E15" t="inlineStr">
@@ -3825,7 +5190,6 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -3861,7 +5225,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="3" t="n">
         <v>46220</v>
       </c>
       <c r="E16" t="inlineStr">
@@ -3874,7 +5238,6 @@
           <t>10:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -3906,7 +5269,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D17" s="3" t="n">
         <v>46224</v>
       </c>
       <c r="E17" t="inlineStr">
@@ -3919,7 +5282,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -3955,7 +5317,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="3" t="n">
         <v>46231</v>
       </c>
       <c r="E18" t="inlineStr">
@@ -3968,7 +5330,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4004,7 +5365,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D19" s="1" t="n">
+      <c r="D19" s="3" t="n">
         <v>46237</v>
       </c>
       <c r="E19" t="inlineStr">
@@ -4017,7 +5378,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4053,7 +5413,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="D20" s="3" t="n">
         <v>46266</v>
       </c>
       <c r="E20" t="inlineStr">
@@ -4066,7 +5426,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4098,7 +5457,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D21" s="1" t="n">
+      <c r="D21" s="3" t="n">
         <v>46279</v>
       </c>
       <c r="E21" t="inlineStr">
@@ -4111,7 +5470,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4147,7 +5505,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D22" s="1" t="n">
+      <c r="D22" s="3" t="n">
         <v>46300</v>
       </c>
       <c r="E22" t="inlineStr">
@@ -4160,7 +5518,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4196,7 +5553,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D23" s="1" t="n">
+      <c r="D23" s="3" t="n">
         <v>46317</v>
       </c>
       <c r="E23" t="inlineStr">
@@ -4209,7 +5566,6 @@
           <t>1:00 PM - 5:00 PM</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4245,7 +5601,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D24" s="1" t="n">
+      <c r="D24" s="3" t="n">
         <v>46328</v>
       </c>
       <c r="E24" t="inlineStr">
@@ -4258,7 +5614,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4294,7 +5649,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D25" s="1" t="n">
+      <c r="D25" s="3" t="n">
         <v>46329</v>
       </c>
       <c r="E25" t="inlineStr">
@@ -4307,7 +5662,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4339,7 +5693,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D26" s="1" t="n">
+      <c r="D26" s="3" t="n">
         <v>46357</v>
       </c>
       <c r="E26" t="inlineStr">
@@ -4352,7 +5706,6 @@
           <t>12:30 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4384,7 +5737,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D27" s="1" t="n">
+      <c r="D27" s="3" t="n">
         <v>46363</v>
       </c>
       <c r="E27" t="inlineStr">
@@ -4397,7 +5750,6 @@
           <t>5:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar *</t>
@@ -4433,7 +5785,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D28" s="1" t="n">
+      <c r="D28" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E28" t="inlineStr">
@@ -4482,7 +5834,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D29" s="1" t="n">
+      <c r="D29" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="E29" t="inlineStr">
@@ -4531,7 +5883,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D30" s="1" t="n">
+      <c r="D30" s="3" t="n">
         <v>46217</v>
       </c>
       <c r="E30" t="inlineStr">
@@ -4580,7 +5932,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D31" s="1" t="n">
+      <c r="D31" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="E31" t="inlineStr">
@@ -4629,7 +5981,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D32" s="1" t="n">
+      <c r="D32" s="3" t="n">
         <v>46216</v>
       </c>
       <c r="E32" t="inlineStr">
@@ -4678,7 +6030,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D33" s="1" t="n">
+      <c r="D33" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E33" t="inlineStr">
@@ -4727,7 +6079,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D34" s="1" t="n">
+      <c r="D34" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E34" t="inlineStr">
@@ -4740,7 +6092,6 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia *</t>
@@ -4772,7 +6123,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D35" s="1" t="n">
+      <c r="D35" s="3" t="n">
         <v>46232</v>
       </c>
       <c r="E35" t="inlineStr">
@@ -4821,7 +6172,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D36" s="1" t="n">
+      <c r="D36" s="3" t="n">
         <v>46206</v>
       </c>
       <c r="E36" t="inlineStr">
@@ -4870,7 +6221,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D37" s="1" t="n">
+      <c r="D37" s="3" t="n">
         <v>46231</v>
       </c>
       <c r="E37" t="inlineStr">
@@ -4919,7 +6270,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D38" s="1" t="n">
+      <c r="D38" s="3" t="n">
         <v>46228</v>
       </c>
       <c r="E38" t="inlineStr">
@@ -4932,7 +6283,6 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia *</t>
@@ -4964,7 +6314,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D39" s="1" t="n">
+      <c r="D39" s="3" t="n">
         <v>46218</v>
       </c>
       <c r="E39" t="inlineStr">
@@ -5013,7 +6363,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D40" s="1" t="n">
+      <c r="D40" s="3" t="n">
         <v>46205</v>
       </c>
       <c r="E40" t="inlineStr">
@@ -5062,7 +6412,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D41" s="1" t="n">
+      <c r="D41" s="3" t="n">
         <v>46224</v>
       </c>
       <c r="E41" t="inlineStr">
@@ -5111,7 +6461,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D42" s="1" t="n">
+      <c r="D42" s="3" t="n">
         <v>46217</v>
       </c>
       <c r="E42" t="inlineStr">
@@ -5160,7 +6510,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D43" s="1" t="n">
+      <c r="D43" s="3" t="n">
         <v>46218</v>
       </c>
       <c r="E43" t="inlineStr">
@@ -5209,7 +6559,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D44" s="1" t="n">
+      <c r="D44" s="3" t="n">
         <v>46225</v>
       </c>
       <c r="E44" t="inlineStr">
@@ -5258,7 +6608,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D45" s="1" t="n">
+      <c r="D45" s="3" t="n">
         <v>46228</v>
       </c>
       <c r="E45" t="inlineStr">
@@ -5307,7 +6657,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D46" s="1" t="n">
+      <c r="D46" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="E46" t="inlineStr">
@@ -5356,7 +6706,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D47" s="1" t="n">
+      <c r="D47" s="3" t="n">
         <v>46232</v>
       </c>
       <c r="E47" t="inlineStr">
@@ -5405,7 +6755,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D48" s="1" t="n">
+      <c r="D48" s="3" t="n">
         <v>46206</v>
       </c>
       <c r="E48" t="inlineStr">
@@ -5454,7 +6804,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D49" s="1" t="n">
+      <c r="D49" s="3" t="n">
         <v>46207</v>
       </c>
       <c r="E49" t="inlineStr">
@@ -5503,7 +6853,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D50" s="1" t="n">
+      <c r="D50" s="3" t="n">
         <v>46207</v>
       </c>
       <c r="E50" t="inlineStr">
@@ -5552,7 +6902,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D51" s="1" t="n">
+      <c r="D51" s="3" t="n">
         <v>46207</v>
       </c>
       <c r="E51" t="inlineStr">
@@ -5601,7 +6951,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D52" s="1" t="n">
+      <c r="D52" s="3" t="n">
         <v>46209</v>
       </c>
       <c r="E52" t="inlineStr">
@@ -5650,7 +7000,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D53" s="1" t="n">
+      <c r="D53" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E53" t="inlineStr">
@@ -5699,7 +7049,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D54" s="1" t="n">
+      <c r="D54" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E54" t="inlineStr">
@@ -5748,7 +7098,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D55" s="1" t="n">
+      <c r="D55" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E55" t="inlineStr">
@@ -5797,7 +7147,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D56" s="1" t="n">
+      <c r="D56" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E56" t="inlineStr">
@@ -5846,7 +7196,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D57" s="1" t="n">
+      <c r="D57" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E57" t="inlineStr">
@@ -5895,7 +7245,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D58" s="1" t="n">
+      <c r="D58" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="E58" t="inlineStr">
@@ -5944,7 +7294,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D59" s="1" t="n">
+      <c r="D59" s="3" t="n">
         <v>46212</v>
       </c>
       <c r="E59" t="inlineStr">
@@ -5993,7 +7343,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D60" s="1" t="n">
+      <c r="D60" s="3" t="n">
         <v>46213</v>
       </c>
       <c r="E60" t="inlineStr">
@@ -6042,7 +7392,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D61" s="1" t="n">
+      <c r="D61" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E61" t="inlineStr">
@@ -6091,7 +7441,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D62" s="1" t="n">
+      <c r="D62" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E62" t="inlineStr">
@@ -6140,7 +7490,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D63" s="1" t="n">
+      <c r="D63" s="3" t="n">
         <v>46218</v>
       </c>
       <c r="E63" t="inlineStr">
@@ -6189,7 +7539,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D64" s="1" t="n">
+      <c r="D64" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="E64" t="inlineStr">
@@ -6238,7 +7588,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D65" s="1" t="n">
+      <c r="D65" s="3" t="n">
         <v>46219</v>
       </c>
       <c r="E65" t="inlineStr">
@@ -6287,7 +7637,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D66" s="1" t="n">
+      <c r="D66" s="3" t="n">
         <v>46220</v>
       </c>
       <c r="E66" t="inlineStr">
@@ -6336,7 +7686,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D67" s="1" t="n">
+      <c r="D67" s="3" t="n">
         <v>46224</v>
       </c>
       <c r="E67" t="inlineStr">
@@ -6385,7 +7735,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D68" s="1" t="n">
+      <c r="D68" s="3" t="n">
         <v>46224</v>
       </c>
       <c r="E68" t="inlineStr">
@@ -6434,7 +7784,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D69" s="1" t="n">
+      <c r="D69" s="3" t="n">
         <v>46224</v>
       </c>
       <c r="E69" t="inlineStr">
@@ -6483,7 +7833,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D70" s="1" t="n">
+      <c r="D70" s="3" t="n">
         <v>46225</v>
       </c>
       <c r="E70" t="inlineStr">
@@ -6532,7 +7882,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D71" s="1" t="n">
+      <c r="D71" s="3" t="n">
         <v>46227</v>
       </c>
       <c r="E71" t="inlineStr">
@@ -6581,7 +7931,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D72" s="1" t="n">
+      <c r="D72" s="3" t="n">
         <v>46231</v>
       </c>
       <c r="E72" t="inlineStr">
@@ -6630,7 +7980,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D73" s="1" t="n">
+      <c r="D73" s="3" t="n">
         <v>46231</v>
       </c>
       <c r="E73" t="inlineStr">
@@ -6679,7 +8029,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D74" s="1" t="n">
+      <c r="D74" s="3" t="n">
         <v>46233</v>
       </c>
       <c r="E74" t="inlineStr">
@@ -6728,7 +8078,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D75" s="1" t="n">
+      <c r="D75" s="3" t="n">
         <v>46240</v>
       </c>
       <c r="E75" t="inlineStr">
@@ -6777,7 +8127,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D76" s="1" t="n">
+      <c r="D76" s="3" t="n">
         <v>46240</v>
       </c>
       <c r="E76" t="inlineStr">
@@ -6826,7 +8176,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D77" s="1" t="n">
+      <c r="D77" s="3" t="n">
         <v>46240</v>
       </c>
       <c r="E77" t="inlineStr">
@@ -6875,7 +8225,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D78" s="1" t="n">
+      <c r="D78" s="3" t="n">
         <v>46245</v>
       </c>
       <c r="E78" t="inlineStr">
@@ -6924,7 +8274,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D79" s="1" t="n">
+      <c r="D79" s="3" t="n">
         <v>46247</v>
       </c>
       <c r="E79" t="inlineStr">
@@ -6973,7 +8323,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D80" s="1" t="n">
+      <c r="D80" s="3" t="n">
         <v>46259</v>
       </c>
       <c r="E80" t="inlineStr">
@@ -7022,7 +8372,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D81" s="1" t="n">
+      <c r="D81" s="3" t="n">
         <v>46261</v>
       </c>
       <c r="E81" t="inlineStr">
@@ -7071,7 +8421,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D82" s="1" t="n">
+      <c r="D82" s="3" t="n">
         <v>46273</v>
       </c>
       <c r="E82" t="inlineStr">
@@ -7120,7 +8470,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D83" s="1" t="n">
+      <c r="D83" s="3" t="n">
         <v>46280</v>
       </c>
       <c r="E83" t="inlineStr">
@@ -7169,7 +8519,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D84" s="1" t="n">
+      <c r="D84" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E84" t="inlineStr">
@@ -7218,7 +8568,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D85" s="1" t="n">
+      <c r="D85" s="3" t="n">
         <v>46249</v>
       </c>
       <c r="E85" t="inlineStr">
@@ -7231,7 +8581,6 @@
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>https://luma.com/genai-collective *</t>
@@ -7263,7 +8612,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D86" s="1" t="n">
+      <c r="D86" s="3" t="n">
         <v>46268</v>
       </c>
       <c r="E86" t="inlineStr">
@@ -7276,7 +8625,6 @@
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>https://luma.com/genai-collective *</t>
@@ -7308,7 +8656,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D87" s="1" t="n">
+      <c r="D87" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E87" t="inlineStr">
@@ -7357,7 +8705,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D88" s="1" t="n">
+      <c r="D88" s="3" t="n">
         <v>46209</v>
       </c>
       <c r="E88" t="inlineStr">
@@ -7406,7 +8754,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D89" s="1" t="n">
+      <c r="D89" s="3" t="n">
         <v>46214</v>
       </c>
       <c r="E89" t="inlineStr">
@@ -7455,7 +8803,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D90" s="1" t="n">
+      <c r="D90" s="3" t="n">
         <v>46228</v>
       </c>
       <c r="E90" t="inlineStr">
@@ -7504,7 +8852,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D91" s="1" t="n">
+      <c r="D91" s="3" t="n">
         <v>46211</v>
       </c>
       <c r="E91" t="inlineStr">
@@ -7553,7 +8901,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D92" s="1" t="n">
+      <c r="D92" s="3" t="n">
         <v>46221</v>
       </c>
       <c r="E92" t="inlineStr">
@@ -7602,7 +8950,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D93" s="1" t="n">
+      <c r="D93" s="3" t="n">
         <v>46221</v>
       </c>
       <c r="E93" t="inlineStr">
@@ -7651,7 +8999,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D94" s="1" t="n">
+      <c r="D94" s="3" t="n">
         <v>46215</v>
       </c>
       <c r="E94" t="inlineStr">
@@ -7700,7 +9048,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D95" s="1" t="n">
+      <c r="D95" s="3" t="n">
         <v>46217</v>
       </c>
       <c r="E95" t="inlineStr">
@@ -7749,7 +9097,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D96" s="1" t="n">
+      <c r="D96" s="3" t="n">
         <v>46224</v>
       </c>
       <c r="E96" t="inlineStr">
@@ -7798,7 +9146,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D97" s="1" t="n">
+      <c r="D97" s="3" t="n">
         <v>46210</v>
       </c>
       <c r="E97" t="inlineStr">
@@ -7851,7 +9199,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D98" s="1" t="n">
+      <c r="D98" s="3" t="n">
         <v>46217</v>
       </c>
       <c r="E98" t="inlineStr">
@@ -7904,7 +9252,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D99" s="1" t="n">
+      <c r="D99" s="3" t="n">
         <v>46217</v>
       </c>
       <c r="E99" t="inlineStr">
@@ -7957,7 +9305,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D100" s="1" t="n">
+      <c r="D100" s="3" t="n">
         <v>46218</v>
       </c>
       <c r="E100" t="inlineStr">
@@ -8010,7 +9358,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D101" s="1" t="n">
+      <c r="D101" s="3" t="n">
         <v>46231</v>
       </c>
       <c r="E101" t="inlineStr">
@@ -8063,7 +9411,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D102" s="1" t="n">
+      <c r="D102" s="3" t="n">
         <v>46233</v>
       </c>
       <c r="E102" t="inlineStr">
@@ -8116,7 +9464,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D103" s="1" t="n">
+      <c r="D103" s="3" t="n">
         <v>46239</v>
       </c>
       <c r="E103" t="inlineStr">
@@ -8169,7 +9517,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D104" s="1" t="n">
+      <c r="D104" s="3" t="n">
         <v>46240</v>
       </c>
       <c r="E104" t="inlineStr">
@@ -8222,7 +9570,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D105" s="1" t="n">
+      <c r="D105" s="3" t="n">
         <v>46244</v>
       </c>
       <c r="E105" t="inlineStr">
@@ -8275,7 +9623,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D106" s="1" t="n">
+      <c r="D106" s="3" t="n">
         <v>46252</v>
       </c>
       <c r="E106" t="inlineStr">
@@ -8328,7 +9676,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D107" s="1" t="n">
+      <c r="D107" s="3" t="n">
         <v>46254</v>
       </c>
       <c r="E107" t="inlineStr">
@@ -8381,7 +9729,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D108" s="1" t="n">
+      <c r="D108" s="3" t="n">
         <v>46268</v>
       </c>
       <c r="E108" t="inlineStr">
@@ -8434,7 +9782,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D109" s="1" t="n">
+      <c r="D109" s="3" t="n">
         <v>46280</v>
       </c>
       <c r="E109" t="inlineStr">
@@ -8487,7 +9835,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D110" s="1" t="n">
+      <c r="D110" s="3" t="n">
         <v>46282</v>
       </c>
       <c r="E110" t="inlineStr">
@@ -8540,7 +9888,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D111" s="1" t="n">
+      <c r="D111" s="3" t="n">
         <v>46289</v>
       </c>
       <c r="E111" t="inlineStr">
@@ -8593,7 +9941,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D112" s="1" t="n">
+      <c r="D112" s="3" t="n">
         <v>46296</v>
       </c>
       <c r="E112" t="inlineStr">
@@ -8646,7 +9994,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D113" s="1" t="n">
+      <c r="D113" s="3" t="n">
         <v>46302</v>
       </c>
       <c r="E113" t="inlineStr">
@@ -8699,7 +10047,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D114" s="1" t="n">
+      <c r="D114" s="3" t="n">
         <v>46310</v>
       </c>
       <c r="E114" t="inlineStr">
@@ -8752,7 +10100,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D115" s="1" t="n">
+      <c r="D115" s="3" t="n">
         <v>46315</v>
       </c>
       <c r="E115" t="inlineStr">
@@ -8805,7 +10153,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D116" s="1" t="n">
+      <c r="D116" s="3" t="n">
         <v>46336</v>
       </c>
       <c r="E116" t="inlineStr">
@@ -8858,7 +10206,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D117" s="1" t="n">
+      <c r="D117" s="3" t="n">
         <v>46338</v>
       </c>
       <c r="E117" t="inlineStr">
@@ -8911,7 +10259,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D118" s="1" t="n">
+      <c r="D118" s="3" t="n">
         <v>46364</v>
       </c>
       <c r="E118" t="inlineStr">
@@ -8964,7 +10312,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D119" s="1" t="n">
+      <c r="D119" s="3" t="n">
         <v>46239</v>
       </c>
       <c r="E119" t="inlineStr">
@@ -9017,7 +10365,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D120" s="1" t="n">
+      <c r="D120" s="3" t="n">
         <v>46246</v>
       </c>
       <c r="E120" t="inlineStr">
@@ -9070,7 +10418,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D121" s="1" t="n">
+      <c r="D121" s="3" t="n">
         <v>46253</v>
       </c>
       <c r="E121" t="inlineStr">
@@ -9123,7 +10471,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D122" s="1" t="n">
+      <c r="D122" s="3" t="n">
         <v>46260</v>
       </c>
       <c r="E122" t="inlineStr">
@@ -9176,7 +10524,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D123" s="1" t="n">
+      <c r="D123" s="3" t="n">
         <v>46267</v>
       </c>
       <c r="E123" t="inlineStr">
@@ -9229,7 +10577,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D124" s="1" t="n">
+      <c r="D124" s="3" t="n">
         <v>46274</v>
       </c>
       <c r="E124" t="inlineStr">
@@ -9282,7 +10630,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D125" s="1" t="n">
+      <c r="D125" s="3" t="n">
         <v>46281</v>
       </c>
       <c r="E125" t="inlineStr">
@@ -9335,7 +10683,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D126" s="1" t="n">
+      <c r="D126" s="3" t="n">
         <v>46288</v>
       </c>
       <c r="E126" t="inlineStr">
@@ -9388,7 +10736,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D127" s="1" t="n">
+      <c r="D127" s="3" t="n">
         <v>46295</v>
       </c>
       <c r="E127" t="inlineStr">
@@ -9441,7 +10789,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D128" s="1" t="n">
+      <c r="D128" s="3" t="n">
         <v>46302</v>
       </c>
       <c r="E128" t="inlineStr">
@@ -9494,7 +10842,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D129" s="1" t="n">
+      <c r="D129" s="3" t="n">
         <v>46306</v>
       </c>
       <c r="E129" t="inlineStr">
@@ -9547,7 +10895,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D130" s="1" t="n">
+      <c r="D130" s="3" t="n">
         <v>46316</v>
       </c>
       <c r="E130" t="inlineStr">
@@ -9600,7 +10948,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D131" s="1" t="n">
+      <c r="D131" s="3" t="n">
         <v>46323</v>
       </c>
       <c r="E131" t="inlineStr">
@@ -9653,7 +11001,7 @@
           <t>high</t>
         </is>
       </c>
-      <c r="D132" s="1" t="n">
+      <c r="D132" s="3" t="n">
         <v>46351</v>
       </c>
       <c r="E132" t="inlineStr">
@@ -9689,6 +11037,1015 @@
       <c r="K132" s="2" t="inlineStr">
         <is>
           <t>The event has zero mention of AI, machine learning, or automation, which is an automatic disqualification regardless of location or format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>IBM SkillsBuild Orientation</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>1</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/ibm-skillsbuild-orientation-1693369?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a mandatory virtual orientation to kick off the upcoming cohort. During this session, participants will receive an overview of the program structure, expectations, key dates, and demo on how to access the learning platform.</t>
+        </is>
+      </c>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>This is a generic orientation/onboarding session with zero mention of AI, machine learning, or automation in its own description, making it an automatic 1 regardless of the hosting organization or platform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>TAG-Ed Pathways to Leadership Virtual Open House</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/qWFX016fkCQCe</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>Join us for an inside look at the Pathways to Leadership program, a year-long leadership experience designed for emerging and mid-level professionals. Learn about the program's structure and benefits and hear from graduates.</t>
+        </is>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the first criterion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>** Canceled ** 2026 Georgia Day of Code</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>1</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="n">
+        <v>46360</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>9:00 AM - 3:00 PM</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/canceled-2026-georgia-day-of-code-1723691?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>2026 Georgia Day of Code is a free, virtual event that introduces computer science and coding skills through engaging learning resources suitable for students of all ages and skill levels.</t>
+        </is>
+      </c>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>Event is canceled and has zero mention of AI, machine learning, or automation in its description, making it an automatic 1 per the primary criterion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Southeastern Hose - Bremen</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>1</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>1:30 PM - 4:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Bremen, Georgia</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/southeastern-hose---bremen</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, which is an automatic 1 regardless of other criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>PAi Manufacturing Facility Tour</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>1</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/ *</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>Get an inside look at one of Georgia's advanced manufacturing operations. The 120,000 sq. ft. production facility features 50 CNC machining centers and 32 industrial robots. Complimentary for AIMST attendees; advance registration required. Space is limited.</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>While the event is in-person in Georgia, it has zero mention of AI, machine learning, or automation in its title and description—it is purely a manufacturing facility tour with no AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>🎬 404 Movie Not Found: Spider-Man (Matinee)</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>1</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>2:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/314126109/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr"/>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is a movie screening event, which triggers the automatic 1 rating regardless of other criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>CISSP Certification Training Course in Bothell, CA</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>1</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Augusta · 22722 29th Dr SE West, Suite 100, Bothell, WA 98021</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/cissp-certification-training-course-in-bothell-ca-tickets-1980894231972?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr"/>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Washington (WA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>The Cost of Bad UX – Based on Real Projects</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>1</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/the-cost-of-bad-ux-based-on-real-projects-tickets-1993809241112?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr"/>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, making it an automatic 1 per the criteria regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Business Analyst (CBAP) Classroom Training in Auburn, AL</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>1</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Columbus · 5547 Veterans Pkwy</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/business-analyst-cbap-classroom-training-in-auburn-al-tickets-1970898472386?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr"/>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation - it is a CBAP (Certified Business Analyst Professional) classroom training course, which is an automatic 1 per the criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Business Analytics Certification (CBAP) Training in Augusta, GA</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Augusta · 823 Broad St</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/business-analytics-certification-cbap-training-in-augusta-ga-tickets-1970052557231?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description - it is a business analytics certification training focused on CBAP (Certified Business Analysis Professional) credential, which is an automatic 1 per the criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Modern Data Architecture 2 Days Training in Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/modern-data-architecture-2-days-training-in-atlanta-ga-tickets-1992366361420?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>The event title and short description contain zero mention of AI, machine learning, or automation, making it an automatic 1 regardless of its in-person Atlanta location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>AWS Solution Architect Training | 4-Day Bootcamp in Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Atlanta · 260 Peachtree St suite 2200</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/aws-solution-architect-training-4-day-bootcamp-in-atlanta-ga-tickets-1987119022488?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr"/>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description - it is purely about AWS Solution Architect certification training, which is a paid training/sales pitch for AWS services rather than an educational AI event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Certified Ethical Hacker – Practical Ethical Hacker in Macon, GA</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Macon · 500a Northside Crossing</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/certified-ethical-hacker-practical-ethical-hacker-in-macon-ga-tickets-1986302519305?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr"/>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is a cybersecurity certification course, which is an automatic 1 per the criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Stronger Communities Through Leadership Skills – 1 Day Training in Atlanta</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Atlanta · Regus - Atlanta - 260 Peachtree</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.sg/e/stronger-communities-through-leadership-skills-1-day-training-in-atlanta-tickets-1702814948349?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of its in-person Atlanta location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Georgia Tech ME 2110 Design Competition: Summer 2026</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Atlanta · Manufacturing Related Disciplines Complex (801 Ferst Dr, Atlanta, GA 30332)</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/georgia-tech-me-2110-design-competition-summer-2026-registration-1991920152798?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr"/>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria regardless of its Georgia Tech in-person location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Naturalist Club: Backyard Habitats &amp; Common Feed Birds</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Kennesaw · North Cobb Regional Library</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/naturalist-club-backyard-habitats-common-feed-birds-tickets-1991154159692?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 per the criteria regardless of its in-person Georgia location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Naturalist Club: Backyard Habitats &amp; Common Feed Birds</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>2:30 PM</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Marietta · East Cobb Library</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/naturalist-club-backyard-habitats-common-feed-birds-tickets-1991153844750?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or in-person status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Naturalist Club: Backyard Habitats &amp; Common Feed Birds</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>1</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>2:30 PM</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Mableton · South Cobb Regional Library</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/naturalist-club-backyard-habitats-common-feed-birds-tickets-1991154120575?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr"/>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation - it is about naturalist club activities and bird watching, which triggers the automatic 1 rating regardless of location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Tech and Wealth Workshop</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>3:00 PM CDT</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1995254351476?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr"/>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering automatic score of 1 per the primary criterion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Bad UX in Numbers: Exploring Real Cases</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="n">
+        <v>46233</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>2:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/bad-ux-in-numbers-exploring-real-cases-tickets-1993810735582?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, making it an automatic 1 regardless of other criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>HIGH-THC Medical Cannabis: A Scientific Breakdown</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>July 27, 2026</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>4:00 PM PDT</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/high-thc-medical-cannabis-a-scientific-breakdown-tickets-1992308768157?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr"/>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation - it is about medical cannabis science, which automatically disqualifies it regardless of other criteria.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-08-03
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K83" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K90" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K153" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K160" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,18 +462,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
@@ -3152,7 +3152,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/MwFNl0es8CeCg</t>
@@ -3197,7 +3196,6 @@
           <t>4:00 PM - 12:30 PM</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/rural-ai-workforce-forum-2026-1759715?sourceTypeId=Website</t>
@@ -3246,7 +3244,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/WqFgM07iaCJCE</t>
@@ -3295,7 +3292,6 @@
           <t>5:00 PM - 7:45 PM</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/xRF50ZqHMCYC7</t>
@@ -3344,7 +3340,6 @@
           <t>6:00 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/EqFedRnCgC6C9</t>
@@ -3393,7 +3388,6 @@
           <t>5:30 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/beyond-connected-iot-s-next-chapter-presented-by-tag-cloud-society-1848946?sourceTypeId=Website</t>
@@ -3442,7 +3436,6 @@
           <t>11:00 AM - 1:30 PM EDT</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/tech-educational-panel</t>
@@ -3482,7 +3475,6 @@
           <t>July 27, 2026</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>Renaissance Atlanta Waverly Hotel &amp; Convention Center, 2450 Galleria Pkwy, Atlanta, GA 30339</t>
@@ -3585,7 +3577,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atl-tech-meetup/events/315779247/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -3679,7 +3670,6 @@
           <t>5:30 PM EDT</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>https://www.meetup.com/aittg-atlanta/events/315755582/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -3822,7 +3812,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atlanta-aws-user-group/events/315805518/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -3846,17 +3835,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" s="3" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
           <t>July 27, 2026</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -3892,7 +3876,6 @@
           <t>9:00 AM EDT</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/building-intelligent-ai-agents-with-graphrag-tickets-1992756563525?aff=ebdssbdestsearch</t>
@@ -3937,7 +3920,6 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/those-time-drains-and-money-leaks-ai-should-be-fixing-that-find-out-how-tickets-1995249007492?aff=ebdssbdestsearch</t>
@@ -4269,8 +4251,6 @@
           <t>July 27, 2026</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-awareness-the-good-the-bad-and-what-to-watch-for-tickets-1991930436557?aff=ebdssbdestsearch</t>
@@ -4315,7 +4295,6 @@
           <t>10:00 AM EDT</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/microsoft-copilot-cowork-masterclass-tickets-1990549050795?aff=ebdssbdestsearch</t>
@@ -4360,7 +4339,6 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-data-analytics-with-genai-bootcamp-usa-only-join-whatsapp-group-tickets-1990886211251?aff=ebdssbdestsearch</t>
@@ -4437,17 +4415,12 @@
           <t>https://www.meetup.com/atlbitlab/events/</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" s="3" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>July 27, 2026</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -4455,6 +4428,241 @@
       </c>
       <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>AIMST - AI Conference - GMA Special Exhibitor and Moderator</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>4</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/aimst---ai-conference---gma-special-exhibitor-and-moderator</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI conference hosted by Georgia Manufacturing Alliance with clear AI focus in title, though specific location within Georgia is missing and description details are sparse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>AnalyticsCLUB JobExpo Virtual Business, Data &amp; Technology Job Expo</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46241</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ac-atl/events/315736240/?recId=8c841573-99a7-4711-95a8-3825b47bc2b0&amp;recSource=ml-popular-events-nearby-online&amp;searchId=1950d877-d2cc-4cf2-979b-834f12b393b2&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>Event has no mention of AI, machine learning, or automation in its title or available description, and while it's hosted by an Atlanta-area organization, the virtual format and lack of AI content trigger the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (AN OPEN AI FORUM FOR ALL)</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>3</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/315016411/?recId=8c841573-99a7-4711-95a8-3825b47bc2b0&amp;recSource=ml-popular-events-nearby-online&amp;searchId=1950d877-d2cc-4cf2-979b-834f12b393b2&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with clear AI focus (Ladies in AI, AI Growth Circle) hosted by a Georgia-based meetup group, but lacks detailed description and is not in-person, limiting its score despite legitimate AI educational content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr"/>
+      <c r="K87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/d/united-states--georgia/science-and-tech--events--this-month/?page=1</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 11, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 34s, resets at Mon Aug 03 2026 17:09:39 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" s="3" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>https://ai.georgia.gov/events</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 12, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 33s, resets at Mon Aug 03 2026 17:09:39 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4470,14 +4678,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K153"/>
+  <dimension ref="A1:K160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -11067,7 +11275,6 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/ibm-skillsbuild-orientation-1693369?sourceTypeId=Website</t>
@@ -11116,7 +11323,6 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/qWFX016fkCQCe</t>
@@ -11165,7 +11371,6 @@
           <t>9:00 AM - 3:00 PM</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/canceled-2026-georgia-day-of-code-1723691?sourceTypeId=Website</t>
@@ -11258,7 +11463,6 @@
           <t>July 27, 2026</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>Georgia</t>
@@ -11312,7 +11516,6 @@
           <t>2:30 PM EDT</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
           <t>https://www.meetup.com/refactr-tech/events/314126109/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -11406,7 +11609,6 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/the-cost-of-bad-ux-based-on-real-projects-tickets-1993809241112?aff=ebdssbdestsearch</t>
@@ -11941,7 +12143,6 @@
           <t>3:00 PM CDT</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1995254351476?aff=ebdssbdestsearch</t>
@@ -11986,7 +12187,6 @@
           <t>2:00 PM EDT</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/bad-ux-in-numbers-exploring-real-cases-tickets-1993810735582?aff=ebdssbdestsearch</t>
@@ -12031,7 +12231,6 @@
           <t>4:00 PM PDT</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/high-thc-medical-cannabis-a-scientific-breakdown-tickets-1992308768157?aff=ebdssbdestsearch</t>
@@ -12046,6 +12245,353 @@
       <c r="K153" s="2" t="inlineStr">
         <is>
           <t>Event has zero mention of AI, machine learning, or automation - it is about medical cannabis science, which automatically disqualifies it regardless of other criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>IBM SkillsBuild Orientation</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/ibm-skillsbuild-orientation-1693369?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a mandatory virtual orientation to kick off the upcoming cohort. During this session, participants will receive an overview of the program structure, expectations, key dates, and a demo on how to access the learning platform.</t>
+        </is>
+      </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation, triggering the automatic-1 rule; it is a generic program orientation with no AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Find a Startup to Help or Join</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="n">
+        <v>46243</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>1:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/projects-for-developers-cs-majors-and-ux-designers/events/315933865/?recId=8c841573-99a7-4711-95a8-3825b47bc2b0&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=1950d877-d2cc-4cf2-979b-834f12b393b2&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr"/>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or available description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Nostr Atlanta #15 - Rush Hour Avoidance</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>4:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>684 John Wesley Dobbs Ave NE suite a1, Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315762247/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>Join us for Nostr Atlanta! Calling all nostr users, content creators, enthusiasts, developers, and more! This session will involve some tool building to avoid rush hour traffic. Informal round-table discussion of Nostr and adjacent topics from 4:30–6:00 PM.</t>
+        </is>
+      </c>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it focuses on Nostr (a decentralized social network protocol) and traffic avoidance, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Manuels Tavern, 602 North Highland Ave NE, Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315044570/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>Join us at Manuel's Tavern for another fun BitPlebs meetup. Casual events geared towards helping you learn about how to get bitcoin, use bitcoin, and understand where it fits into current events. Arrive early for some free beverages. Agenda includes kick-off, community announcements, a presentation, and a beer social.</t>
+        </is>
+      </c>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is exclusively about Bitcoin and cryptocurrency education, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Manuel's Tavern, 602 North Highland Avenue Northeast, Atlanta, GA 30307</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315044571/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr"/>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of location or in-person status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Manuel's Tavern, 602 North Highland Avenue Northeast, Atlanta, GA 30307</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315044572/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr"/>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or in-person status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>46351</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>August 3, 2026</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>6:00 PM EST</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Manuel's Tavern, 602 North Highland Avenue Northeast, Atlanta, GA 30307</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315044573/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of location or format.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert master to pre-2026-08-03 state
The 2026-08-03 run hit Firecrawl rate limits on 2 of 10 sites, so its
events_master.xlsx additions are being rolled back to last week's
(2026-07-27) state before the next scheduled run.
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K90" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K83" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K160" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K153" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,18 +462,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
@@ -3152,6 +3152,7 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/MwFNl0es8CeCg</t>
@@ -3196,6 +3197,7 @@
           <t>4:00 PM - 12:30 PM</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/rural-ai-workforce-forum-2026-1759715?sourceTypeId=Website</t>
@@ -3244,6 +3246,7 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/WqFgM07iaCJCE</t>
@@ -3292,6 +3295,7 @@
           <t>5:00 PM - 7:45 PM</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/xRF50ZqHMCYC7</t>
@@ -3340,6 +3344,7 @@
           <t>6:00 PM - 7:30 PM</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/EqFedRnCgC6C9</t>
@@ -3388,6 +3393,7 @@
           <t>5:30 PM - 8:00 PM</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/beyond-connected-iot-s-next-chapter-presented-by-tag-cloud-society-1848946?sourceTypeId=Website</t>
@@ -3436,6 +3442,7 @@
           <t>11:00 AM - 1:30 PM EDT</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/tech-educational-panel</t>
@@ -3475,6 +3482,7 @@
           <t>July 27, 2026</t>
         </is>
       </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>Renaissance Atlanta Waverly Hotel &amp; Convention Center, 2450 Galleria Pkwy, Atlanta, GA 30339</t>
@@ -3577,6 +3585,7 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atl-tech-meetup/events/315779247/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -3670,6 +3679,7 @@
           <t>5:30 PM EDT</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>https://www.meetup.com/aittg-atlanta/events/315755582/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -3812,6 +3822,7 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atlanta-aws-user-group/events/315805518/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -3835,12 +3846,17 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
       <c r="D70" s="3" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
           <t>July 27, 2026</t>
         </is>
       </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -3876,6 +3892,7 @@
           <t>9:00 AM EDT</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/building-intelligent-ai-agents-with-graphrag-tickets-1992756563525?aff=ebdssbdestsearch</t>
@@ -3920,6 +3937,7 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/those-time-drains-and-money-leaks-ai-should-be-fixing-that-find-out-how-tickets-1995249007492?aff=ebdssbdestsearch</t>
@@ -4251,6 +4269,8 @@
           <t>July 27, 2026</t>
         </is>
       </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-awareness-the-good-the-bad-and-what-to-watch-for-tickets-1991930436557?aff=ebdssbdestsearch</t>
@@ -4295,6 +4315,7 @@
           <t>10:00 AM EDT</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/microsoft-copilot-cowork-masterclass-tickets-1990549050795?aff=ebdssbdestsearch</t>
@@ -4339,6 +4360,7 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-data-analytics-with-genai-bootcamp-usa-only-join-whatsapp-group-tickets-1990886211251?aff=ebdssbdestsearch</t>
@@ -4415,12 +4437,17 @@
           <t>https://www.meetup.com/atlbitlab/events/</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
       <c r="D83" s="3" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
           <t>July 27, 2026</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -4428,241 +4455,6 @@
       </c>
       <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>AIMST - AI Conference - GMA Special Exhibitor and Moderator</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>4</v>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="n">
-        <v>46252</v>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>https://www.georgiamanufacturingalliance.com/events/aimst---ai-conference---gma-special-exhibitor-and-moderator</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J84" s="2" t="inlineStr"/>
-      <c r="K84" s="2" t="inlineStr">
-        <is>
-          <t>In-person AI conference hosted by Georgia Manufacturing Alliance with clear AI focus in title, though specific location within Georgia is missing and description details are sparse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>AnalyticsCLUB JobExpo Virtual Business, Data &amp; Technology Job Expo</t>
-        </is>
-      </c>
-      <c r="B85" t="n">
-        <v>1</v>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="n">
-        <v>46241</v>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>11:00 AM EDT</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/ac-atl/events/315736240/?recId=8c841573-99a7-4711-95a8-3825b47bc2b0&amp;recSource=ml-popular-events-nearby-online&amp;searchId=1950d877-d2cc-4cf2-979b-834f12b393b2&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J85" s="2" t="inlineStr"/>
-      <c r="K85" s="2" t="inlineStr">
-        <is>
-          <t>Event has no mention of AI, machine learning, or automation in its title or available description, and while it's hosted by an Atlanta-area organization, the virtual format and lack of AI content trigger the automatic-1 rule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (AN OPEN AI FORUM FOR ALL)</t>
-        </is>
-      </c>
-      <c r="B86" t="n">
-        <v>3</v>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D86" s="3" t="n">
-        <v>46240</v>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>7:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/ai-growth-circle/events/315016411/?recId=8c841573-99a7-4711-95a8-3825b47bc2b0&amp;recSource=ml-popular-events-nearby-online&amp;searchId=1950d877-d2cc-4cf2-979b-834f12b393b2&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J86" s="2" t="inlineStr"/>
-      <c r="K86" s="2" t="inlineStr">
-        <is>
-          <t>Virtual-only event with clear AI focus (Ladies in AI, AI Growth Circle) hosted by a Georgia-based meetup group, but lacks detailed description and is not in-person, limiting its score despite legitimate AI educational content.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>https://luma.com/genai-collective</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" s="3" t="inlineStr"/>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>no_events</t>
-        </is>
-      </c>
-      <c r="J87" s="2" t="inlineStr"/>
-      <c r="K87" s="2" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>https://www.eventbrite.com/d/united-states--georgia/science-and-tech--events--this-month/?page=1</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
-      <c r="D88" s="3" t="inlineStr"/>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 11, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 34s, resets at Mon Aug 03 2026 17:09:39 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
-        </is>
-      </c>
-      <c r="J88" s="2" t="inlineStr"/>
-      <c r="K88" s="2" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>https://atlanta.aitinkerers.org/</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" s="3" t="inlineStr"/>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>no_events</t>
-        </is>
-      </c>
-      <c r="J89" s="2" t="inlineStr"/>
-      <c r="K89" s="2" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>https://ai.georgia.gov/events</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
-      <c r="D90" s="3" t="inlineStr"/>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 12, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 33s, resets at Mon Aug 03 2026 17:09:39 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
-        </is>
-      </c>
-      <c r="J90" s="2" t="inlineStr"/>
-      <c r="K90" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4678,14 +4470,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K160"/>
+  <dimension ref="A1:K153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -11275,6 +11067,7 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/ibm-skillsbuild-orientation-1693369?sourceTypeId=Website</t>
@@ -11323,6 +11116,7 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/qWFX016fkCQCe</t>
@@ -11371,6 +11165,7 @@
           <t>9:00 AM - 3:00 PM</t>
         </is>
       </c>
+      <c r="G135" t="inlineStr"/>
       <c r="H135" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/canceled-2026-georgia-day-of-code-1723691?sourceTypeId=Website</t>
@@ -11463,6 +11258,7 @@
           <t>July 27, 2026</t>
         </is>
       </c>
+      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>Georgia</t>
@@ -11516,6 +11312,7 @@
           <t>2:30 PM EDT</t>
         </is>
       </c>
+      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
           <t>https://www.meetup.com/refactr-tech/events/314126109/?recId=0ebce766-0208-4387-bd1d-76e940ebf82c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=05035234-c275-48f4-b199-f583ac5b76b3&amp;eventOrigin=find_page%24all</t>
@@ -11609,6 +11406,7 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
+      <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/the-cost-of-bad-ux-based-on-real-projects-tickets-1993809241112?aff=ebdssbdestsearch</t>
@@ -12143,6 +11941,7 @@
           <t>3:00 PM CDT</t>
         </is>
       </c>
+      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1995254351476?aff=ebdssbdestsearch</t>
@@ -12187,6 +11986,7 @@
           <t>2:00 PM EDT</t>
         </is>
       </c>
+      <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/bad-ux-in-numbers-exploring-real-cases-tickets-1993810735582?aff=ebdssbdestsearch</t>
@@ -12231,6 +12031,7 @@
           <t>4:00 PM PDT</t>
         </is>
       </c>
+      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/high-thc-medical-cannabis-a-scientific-breakdown-tickets-1992308768157?aff=ebdssbdestsearch</t>
@@ -12245,353 +12046,6 @@
       <c r="K153" s="2" t="inlineStr">
         <is>
           <t>Event has zero mention of AI, machine learning, or automation - it is about medical cannabis science, which automatically disqualifies it regardless of other criteria.</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>IBM SkillsBuild Orientation</t>
-        </is>
-      </c>
-      <c r="B154" t="n">
-        <v>1</v>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D154" s="3" t="n">
-        <v>46260</v>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>6:00 PM - 7:00 PM</t>
-        </is>
-      </c>
-      <c r="G154" t="inlineStr"/>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>https://members.tagonline.org/calendar/Details/ibm-skillsbuild-orientation-1693369?sourceTypeId=Website</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J154" s="2" t="inlineStr">
-        <is>
-          <t>Join us for a mandatory virtual orientation to kick off the upcoming cohort. During this session, participants will receive an overview of the program structure, expectations, key dates, and a demo on how to access the learning platform.</t>
-        </is>
-      </c>
-      <c r="K154" s="2" t="inlineStr">
-        <is>
-          <t>The event description contains zero mention of AI, machine learning, or automation, triggering the automatic-1 rule; it is a generic program orientation with no AI-focused component.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Find a Startup to Help or Join</t>
-        </is>
-      </c>
-      <c r="B155" t="n">
-        <v>1</v>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D155" s="3" t="n">
-        <v>46243</v>
-      </c>
-      <c r="E155" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F155" t="inlineStr">
-        <is>
-          <t>1:30 PM EDT</t>
-        </is>
-      </c>
-      <c r="G155" t="inlineStr"/>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/projects-for-developers-cs-majors-and-ux-designers/events/315933865/?recId=8c841573-99a7-4711-95a8-3825b47bc2b0&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=1950d877-d2cc-4cf2-979b-834f12b393b2&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I155" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J155" s="2" t="inlineStr"/>
-      <c r="K155" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or available description, triggering the automatic-1 rule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Nostr Atlanta #15 - Rush Hour Avoidance</t>
-        </is>
-      </c>
-      <c r="B156" t="n">
-        <v>1</v>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D156" s="3" t="n">
-        <v>46253</v>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr">
-        <is>
-          <t>4:30 PM EDT</t>
-        </is>
-      </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>684 John Wesley Dobbs Ave NE suite a1, Atlanta, GA, US</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/atlbitlab/events/315762247/?eventOrigin=group_events_list</t>
-        </is>
-      </c>
-      <c r="I156" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J156" s="2" t="inlineStr">
-        <is>
-          <t>Join us for Nostr Atlanta! Calling all nostr users, content creators, enthusiasts, developers, and more! This session will involve some tool building to avoid rush hour traffic. Informal round-table discussion of Nostr and adjacent topics from 4:30–6:00 PM.</t>
-        </is>
-      </c>
-      <c r="K156" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it focuses on Nostr (a decentralized social network protocol) and traffic avoidance, triggering the automatic-1 rule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
-        </is>
-      </c>
-      <c r="B157" t="n">
-        <v>1</v>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D157" s="3" t="n">
-        <v>46260</v>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr">
-        <is>
-          <t>6:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>Manuels Tavern, 602 North Highland Ave NE, Atlanta, GA, US</t>
-        </is>
-      </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/atlbitlab/events/315044570/?eventOrigin=group_events_list</t>
-        </is>
-      </c>
-      <c r="I157" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J157" s="2" t="inlineStr">
-        <is>
-          <t>Join us at Manuel's Tavern for another fun BitPlebs meetup. Casual events geared towards helping you learn about how to get bitcoin, use bitcoin, and understand where it fits into current events. Arrive early for some free beverages. Agenda includes kick-off, community announcements, a presentation, and a beer social.</t>
-        </is>
-      </c>
-      <c r="K157" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is exclusively about Bitcoin and cryptocurrency education, triggering the automatic-1 rule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
-        </is>
-      </c>
-      <c r="B158" t="n">
-        <v>1</v>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D158" s="3" t="n">
-        <v>46288</v>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>6:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>Manuel's Tavern, 602 North Highland Avenue Northeast, Atlanta, GA 30307</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/atlbitlab/events/315044571/?eventOrigin=group_events_list</t>
-        </is>
-      </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J158" s="2" t="inlineStr"/>
-      <c r="K158" s="2" t="inlineStr">
-        <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of location or in-person status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
-        </is>
-      </c>
-      <c r="B159" t="n">
-        <v>1</v>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D159" s="3" t="n">
-        <v>46323</v>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>6:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>Manuel's Tavern, 602 North Highland Avenue Northeast, Atlanta, GA 30307</t>
-        </is>
-      </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/atlbitlab/events/315044572/?eventOrigin=group_events_list</t>
-        </is>
-      </c>
-      <c r="I159" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J159" s="2" t="inlineStr"/>
-      <c r="K159" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or in-person status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - June</t>
-        </is>
-      </c>
-      <c r="B160" t="n">
-        <v>1</v>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D160" s="3" t="n">
-        <v>46351</v>
-      </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>August 3, 2026</t>
-        </is>
-      </c>
-      <c r="F160" t="inlineStr">
-        <is>
-          <t>6:00 PM EST</t>
-        </is>
-      </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>Manuel's Tavern, 602 North Highland Avenue Northeast, Atlanta, GA 30307</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/atlbitlab/events/315044573/?eventOrigin=group_events_list</t>
-        </is>
-      </c>
-      <c r="I160" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J160" s="2" t="inlineStr"/>
-      <c r="K160" s="2" t="inlineStr">
-        <is>
-          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of location or format.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-08-10
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K118" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K140" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K204" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K215" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,14 +462,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -4456,7 +4456,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
           <t>https://www.meetup.com/modernwebatl/events/315488146/?recId=c9fa2fcb-2337-495c-ac93-1d91a25e8b54&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=0500200c-b3c2-429f-8698-91ed31868873&amp;eventOrigin=find_page%24all</t>
@@ -4501,7 +4500,6 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>https://www.meetup.com/freeside-atlanta/events/315410843/?recId=c9fa2fcb-2337-495c-ac93-1d91a25e8b54&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=0500200c-b3c2-429f-8698-91ed31868873&amp;eventOrigin=find_page%24all</t>
@@ -4525,17 +4523,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" s="3" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>August 3, 2026</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -4571,7 +4564,6 @@
           <t>2:00 PM CDT</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1996426857473?aff=ebdssbdestsearch</t>
@@ -4910,7 +4902,6 @@
           <t>3:00 PM CDT</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1996426541528?aff=ebdssbdestsearch</t>
@@ -4955,7 +4946,6 @@
           <t>9:30 AM EDT</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/machine-learning-for-trading-in-the-age-of-ai-agents-tickets-1994299755253?aff=ebdssbdestsearch</t>
@@ -5392,7 +5382,6 @@
           <t>10:00 AM EDT</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/build-executive-ready-excel-reports-with-microsoft-copilot-tickets-1994204467244?aff=ebdssbdestsearch</t>
@@ -5479,8 +5468,6 @@
           <t>August 3, 2026</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/part-2-make-sense-of-information-ai-for-reading-research-documents-tickets-1990585353377?aff=ebdssbdestsearch</t>
@@ -5525,7 +5512,6 @@
           <t>11:00 AM</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-for-job-seekers-tickets-1994096418066?aff=ebdssbdestsearch</t>
@@ -5717,7 +5703,6 @@
           <t>2:00 PM CDT</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1996425661897?aff=ebdssbdestsearch</t>
@@ -5839,17 +5824,12 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
-      <c r="C114" t="inlineStr"/>
       <c r="D114" s="3" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
           <t>August 3, 2026</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -5885,7 +5865,6 @@
           <t>11:00 a.m.</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
           <t>https://ai.georgia.gov/events/2026-08-06/role-based-training-chatgpt-it-security-teams</t>
@@ -5930,7 +5909,6 @@
           <t>2:30 p.m.</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
           <t>https://ai.georgia.gov/events/2026-08-17/chatgpt-project-and-program-managers</t>
@@ -5975,7 +5953,6 @@
           <t>1:30 p.m.</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
           <t>https://ai.georgia.gov/events/2026-08-25/chatgpt-essentials</t>
@@ -6039,6 +6016,1040 @@
       <c r="K118" s="2" t="inlineStr">
         <is>
           <t>In-person Atlanta event hosted by Georgia's official AI organization with a clear data-driven/AI focus in the title, but the empty description prevents full assessment of content depth and whether it's educational or sales-oriented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>How AI Is Supercharging NextGen Solutions and the Investing Landscape presented by TAG Corporate Development Society and TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>2</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>5:30 PM - 8:30 PM</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/4lFXlWOiRCMCx</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>Sharp insight from the executives living this shift firsthand, and a front-row seat to the founders building next gen solutions.</t>
+        </is>
+      </c>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>Event has genuine AI content (TAG Data Science &amp; AI Society is a co-host with stated AI focus) but is virtual-only with no clear Georgia organizational tie, and the vague description lacks specific session details about the AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Data Ingestion in Fabric - Ginger Grant</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>1</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/dba-fundamentals-group/events/315182870/?recId=638524a7-d934-4434-9d4f-83e72a5d59ae&amp;recSource=ml-popular-events-nearby-online&amp;searchId=e8c9bfc6-65cd-4d6d-af2f-2539b9217477&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr"/>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>Event has no mention of AI, machine learning, or automation in its title or available description, and appears to be a technical data/database session rather than AI-focused content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Meet Atlanta Tech Week &amp; RenderATL Speakers! **JOIN WAITLIST ON LUMA)**</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>1</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/315473059/?recId=638524a7-d934-4434-9d4f-83e72a5d59ae&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=e8c9bfc6-65cd-4d6d-af2f-2539b9217477&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr"/>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>Event has no description content and title mentions only a speaker meetup with no indication of AI, machine learning, or automation focus, making it impossible to verify AI relevance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (AN OPEN AI FORUM FOR ALL)</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>2</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/315016426/?recId=638524a7-d934-4434-9d4f-83e72a5d59ae&amp;recSource=ml-popular-events-nearby-online&amp;searchId=e8c9bfc6-65cd-4d6d-af2f-2539b9217477&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with AI focus (Ladies in AI + AI Growth Circle) but no Georgia organizational tie mentioned, no detailed description provided, and online format limits its value for a Georgia-focused digest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr"/>
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" s="3" t="inlineStr"/>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr"/>
+      <c r="K123" s="2" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Health &amp; Life Sciences Research Tech</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>1</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/health-life-sciences-research-tech-tickets-1990892797952?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>Event details lack any mention of AI, machine learning, or automation in the title or description, and the empty short description prevents assessment of genuine AI-focused content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>AI Literacy Bootcamp</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>2</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-literacy-bootcamp-tickets-1997208273710?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr"/>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>Event has clear AI content in title but is virtual-only with no Georgia organizational tie mentioned, and critical details like description and host organization are missing, making it impossible to verify Georgia focus or assess educational quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>The Future Is Here! AI 2026: What's New, What's Next &amp; What Matters!</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>4</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Eatonton · 951 Harmony Rd suite 102</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/the-future-is-here-ai-2026-whats-new-whats-next-what-matters-tickets-1996530858543?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>In-person event in Eatonton (outside metro Atlanta) with clear AI focus in title, but empty description limits confidence in assessing event quality and depth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Strategic Prompt Design for AI 1 Day Training in Marietta, GA</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>2</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Marietta, GA</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/strategic-prompt-design-for-ai-1-day-training-in-marietta-ga-tickets-1992104255454?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr"/>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>Event is in-person in Georgia (positive), has AI content in title, but appears to be a paid training/sales pitch with no description provided to assess educational value or legitimacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Summer Connections: Atlanta Tech Week Edition</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>1</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Atlanta · High Society Buckhead</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/summer-connections-atlanta-tech-week-edition-tickets-1997135499039?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr"/>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule, though the extremely sparse details (missing description) prevent higher confidence in this assessment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Curiosity Night at Laurel and Lore</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>1</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Guyton · 181 Old Oak Rd</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/curiosity-night-at-laurel-and-lore-tickets-1997333264561?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr"/>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule despite being in-person in Georgia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>4-Day Data Science with Python Bootcamp in Macon, GA</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>3</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Fayetteville · 320 W Lanier Ave</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/4-day-data-science-with-python-bootcamp-in-macon-ga-tickets-1985401411066?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>In-person data science bootcamp in Georgia (Fayetteville, near Macon) with clear AI/machine learning relevance, but lacks detailed description and appears to be a paid training program which scores moderately rather than highly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Data Science with Phython Certification Training in Columbus, GA</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>2</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Columbus · 5547 Veterans Pkwy</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/data-science-with-phython-certification-training-in-columbus-ga-tickets-1985087343682?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr"/>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>While this is an in-person event in Columbus, GA (outside metro Atlanta, which is positive), it appears to be a paid certification training course that is likely a sales-focused offering rather than an educational AI event, and the description lacks any specific mention of AI, machine learning, or automation components despite being data science training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Data Science with Python Certification Training in Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>2</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Atlanta · 3423 Piedmont Rd NE</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/data-science-with-python-certification-training-in-atlanta-ga-tickets-1984745299619?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr"/>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>Event is in-person in Atlanta with potential AI relevance (data science), but the complete absence of description and heavy emphasis on 'certification training' suggests it may be a paid training/sales pitch rather than an educational conference, and the lack of detail prevents confident assessment of its AI content quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>How to Get Started with Artificial Intelligence (AI)</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>4</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Marietta · Switzer Library</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/how-to-get-started-with-artificial-intelligence-ai-tickets-1993857732150?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr"/>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI event in Marietta (outside Atlanta metro) with clear AI focus in title, though empty description limits confidence and suggests it may be a basic introductory session rather than in-depth technical content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>AARI x Waymo x Chic-Fil-a Back to School Robotics Event (In Person)</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>4</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Atlanta · Russell Innovation Center for Entrepreneurs</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/aari-x-waymo-x-chic-fil-a-back-to-school-robotics-event-in-person-tickets-1997019634485?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>In-person Atlanta robotics event with clear AI/automation focus (Waymo autonomous vehicles partnership) and educational mission, though the empty description limits confidence in assessing depth of AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Wednesd.AI</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>4</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Atlanta · Atlanta Tech Village - Buckhead</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr"/>
+      <c r="K135" s="2" t="inlineStr">
+        <is>
+          <t>In-person Atlanta event with clear AI focus in title (Wednesd.AI), but confidence is medium due to missing event description that would clarify the specific AI content and format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>AI Awareness: The Good, the Bad, and What to Watch For</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>4</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>East Point · 1928 Stanton Rd</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-awareness-the-good-the-bad-and-what-to-watch-for-tickets-1991930436557?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>In-person event in Georgia (East Point) with clear AI focus in title and theme, though limited description details prevent a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>AI Training for Business Owners: Get Out of the Day-to-Day (Free, Live)</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>2</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-training-for-business-owners-get-out-of-the-day-to-day-free-live-tickets-1996472647432?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr"/>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Event has clear AI content in title but is virtual-only with no Georgia organizational tie evident, no location specified, and appears to be a free business training that could be a sales pitch, warranting a low score pending more information.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>AI Tinkerers Atlanta x AI Collective: Community Demos at ATL Tech Week</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>4</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>1:45 PM EDT</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/p/ai-tinkerers-atlanta-x-ai-collective-community-demos-at-atl-tech-week</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>AI Tinkerers Atlanta and AI Collective will host community demos. Sponsors AI Collective and Atlanta Tech Week will support the event.</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI-focused community event in Atlanta with clear AI content (demos) hosted by established AI organizations, though the brief description lacks specific session details that would warrant a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Role Based Training: ChatGPT for Procurement</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>4</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>11:00 a.m.</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>https://ai.georgia.gov/events/2026-08-24/chatgpt-procurement</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr"/>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>AI-focused training event (ChatGPT) hosted by Georgia's official AI organization (ai.georgia.gov) with clear Georgia tie, but virtual format and lack of description details prevent higher rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>ChatGPT Advanced Use</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>3</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="n">
+        <v>46267</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>10:00 a.m.</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>https://ai.georgia.gov/events/2026-09-02/chatgpt-advanced-use</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr"/>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>The event has clear AI content (ChatGPT) and is hosted by ai.georgia.gov, a Georgia-based organization, which elevates a virtual-only event to the 3-4 range, but the lack of description and details prevents a higher score.</t>
         </is>
       </c>
     </row>
@@ -6056,14 +7067,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K204"/>
+  <dimension ref="A1:K215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -13653,7 +14664,6 @@
           <t>5:30 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/4lFO0aGuRCMCx</t>
@@ -13702,7 +14712,6 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/ibm-skillsbuild-orientation-1693369?sourceTypeId=Website</t>
@@ -13751,7 +14760,6 @@
           <t>1:30 PM EDT</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
           <t>https://www.meetup.com/projects-for-developers-cs-majors-and-ux-designers/events/315933865/?recId=c9fa2fcb-2337-495c-ac93-1d91a25e8b54&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=0500200c-b3c2-429f-8698-91ed31868873&amp;eventOrigin=find_page%24all</t>
@@ -15063,7 +16071,6 @@
           <t>August 3, 2026</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>Athens, GA</t>
@@ -15505,7 +16512,6 @@
           <t>1:00 PM</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/stay-safe-online-cybersecurity-for-seniors-tickets-1992514958879?aff=ebdssbdestsearch</t>
@@ -15648,7 +16654,6 @@
           <t>6:30 PM</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/stormwater-education-program-tickets-1995485724519?aff=ebdssbdestsearch</t>
@@ -15693,7 +16698,6 @@
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/great-pollinator-census-tickets-1995488467724?aff=ebdssbdestsearch</t>
@@ -15787,7 +16791,6 @@
           <t>4:00 PM</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/gmail-basics-tickets-1993856585721?aff=ebdssbdestsearch</t>
@@ -15832,7 +16835,6 @@
           <t>6:30 PM</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/georgia-adopt-a-stream-chemical-monitoring-workshop-tickets-1970640942106?aff=ebdssbdestsearch</t>
@@ -16100,6 +17102,531 @@
       <c r="K204" s="2" t="inlineStr">
         <is>
           <t>Event has zero mention of AI, machine learning, or automation in title or description, triggering the automatic-1 rule despite being in-person in Atlanta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Hacking the System: Health, Freedom and Income</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>1</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr"/>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/hacking-the-system-health-freedom-and-income-tickets-1994593661334?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr"/>
+      <c r="K205" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Business Analyst (CBAP) Classroom Training in Athens, GA</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>1</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Athens · 2470 Daniells Bridge Rd</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/business-analyst-cbap-classroom-training-in-athens-ga-tickets-1970897699073?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr"/>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description - it is a business analyst certification training course with no AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>STEM Family Sundays at iFLY Atlanta!</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>1</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="n">
+        <v>46264</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Atlanta · iFLY Indoor Skydiving - Atlanta</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/stem-family-sundays-at-ifly-atlanta-tickets-1991765472144?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr"/>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or available description, triggering the automatic-1 rule regardless of in-person Atlanta location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Composting 101 Workshop with Green Done Wright</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>1</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Avondale Estates · 32 N Avondale Rd suite c</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/composting-101-workshop-with-green-done-wright-tickets-1996638381146?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr"/>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation - it is a composting workshop with no AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>CEH Certification In-Person Training in Augusta, GA</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>1</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Augusta, GA</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ceh-certification-in-person-training-in-augusta-ga-tickets-1986891577193?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr"/>
+      <c r="K209" s="2" t="inlineStr">
+        <is>
+          <t>CEH (Certified Ethical Hacker) certification training has no mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of its in-person Georgia location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>CEH Certification Weekend Training Course in Savannah, GA</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>1</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr"/>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Savannah, GA</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ceh-certification-weekend-training-course-in-savannah-ga-tickets-1986878155047?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr"/>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or available description - it is a CEH (Certified Ethical Hacker) certification course focused on cybersecurity, not AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>CEH v12 Ethical Hacking Bootcamp – 4 Days Training in Athens, GA</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>1</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Athens · 2470 Daniells Bridge Rd Building 100 / Suite 161, Athens, GA 30606</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ceh-v12-ethical-hacking-bootcamp-4-days-training-in-athens-ga-tickets-1986397488360?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr"/>
+      <c r="K211" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is purely about ethical hacking certification training, which is a cybersecurity topic distinct from AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>AWS Solution Architect Training in Athens, GA</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>1</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Athens, GA</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/aws-solution-architect-training-in-athens-ga-tickets-1987328746779?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr"/>
+      <c r="K212" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule despite being in-person in Georgia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>AWS Solutions Architect Associate Certification Training in Augusta, GA</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>1</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr"/>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Augusta, GA</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/aws-solutions-architect-associate-certification-training-in-augusta-ga-tickets-1987307393912?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr"/>
+      <c r="K213" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is AWS certification training content with no stated AI-focused component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>CISSP Certification Weekend Training Course in Savannah, GA</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>1</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Savannah · Gallo Legal Services Savannah</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/cissp-certification-weekend-training-course-in-savannah-ga-tickets-1981281933598?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr"/>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is a CISSP cybersecurity certification training course with no AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>CISSP Certification | ISC² Exam Preparation Program in Columbus, GA</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>1</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>August 10, 2026</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Columbus, GA</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/cissp-certification-isc2-exam-preparation-program-in-columbus-ga-tickets-1980702995980?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr"/>
+      <c r="K215" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation—it is a CISSP cybersecurity certification exam prep program with no AI-focused component.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-08-17
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K140" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K166" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K215" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K243" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K140"/>
+  <dimension ref="A1:K166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -6046,7 +6046,6 @@
           <t>5:30 PM - 8:30 PM</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
       <c r="H119" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/4lFXlWOiRCMCx</t>
@@ -6144,7 +6143,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
           <t>https://www.meetup.com/refactr-tech/events/315473059/?recId=638524a7-d934-4434-9d4f-83e72a5d59ae&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=e8c9bfc6-65cd-4d6d-af2f-2539b9217477&amp;eventOrigin=find_page%24all</t>
@@ -6217,17 +6215,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
       <c r="D123" s="3" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
           <t>August 10, 2026</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -6263,7 +6256,6 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/health-life-sciences-research-tech-tickets-1990892797952?aff=ebdssbdestsearch</t>
@@ -6308,7 +6300,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-literacy-bootcamp-tickets-1997208273710?aff=ebdssbdestsearch</t>
@@ -6892,7 +6883,6 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-training-for-business-owners-get-out-of-the-day-to-day-free-live-tickets-1996472647432?aff=ebdssbdestsearch</t>
@@ -6990,7 +6980,6 @@
           <t>11:00 a.m.</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
           <t>https://ai.georgia.gov/events/2026-08-24/chatgpt-procurement</t>
@@ -7035,7 +7024,6 @@
           <t>10:00 a.m.</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr">
         <is>
           <t>https://ai.georgia.gov/events/2026-09-02/chatgpt-advanced-use</t>
@@ -7052,6 +7040,1186 @@
           <t>The event has clear AI content (ChatGPT) and is hosted by ai.georgia.gov, a Georgia-based organization, which elevates a virtual-only event to the 3-4 range, but the lack of description and details prevents a higher score.</t>
         </is>
       </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Data Center Bus Tour presented by TAG Infrastructure Society</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>1</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>8:30 AM - 2:00 PM</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/qWFJmQmFkCQCe</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr"/>
+      <c r="K141" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or available description, triggering the automatic-1 rule despite being in-person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>AIMST - AI Conference - GMA Special Exhibitor and Moderator</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>4</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/aimst---ai-conference---gma-special-exhibitor-and-moderator</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI conference with Georgia manufacturing industry tie (GMA = Georgia Manufacturing Alliance), though the minimal event description and missing location details prevent a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>**New location** 🎬 404 Movie Not Found: Coyote vs. Acme</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="n">
+        <v>46263</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>4:20 PM EDT</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/315951068/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>Event title and description contain no mention of AI, machine learning, or automation, and the empty short description provides no additional context to indicate AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Building AI-Ready Teams — Talent, Culture &amp; Leadership in the AI Era</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>4</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>5:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316063226/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr"/>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI-focused title and Georgia AI Alliance hosting indicate genuine AI content, in-person format is favorable, but missing location details and empty description prevent higher confidence and optimal scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Open House!</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>7:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/freeside-atlanta/events/315371013/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr"/>
+      <c r="K145" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule despite being in-person and hosted by Freeside Atlanta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>GA AI Alliance Networking Lunch</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>3</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>11:45 AM EDT</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/315873146/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>Event is in-person and hosted by Georgia AI Alliance (Georgia-based org) which strongly suggests AI focus, but the completely empty description and lack of specific AI content details in the listing prevent a higher confidence score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Kiro Workshop: Let's Finish What We Started!</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlanta-aws-user-group/events/316120191/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-online&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr"/>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>Event has no description and title provides no indication of AI, machine learning, or automation content, making it impossible to assess the AI component despite being hosted by an AWS user group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>BHS X Sandbox Atlanta Present: CTF Training for First-timers</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/blackhack-society-atlanta/events/315951497/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>Event has no mention of AI, machine learning, or automation in its title or available description, and CTF (Capture The Flag) training is a cybersecurity competition skill unrelated to AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Power of the Noun: Intro to IA in the Age of AI</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>3</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ladies-that-ux-atl/events/314440739/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>The event title explicitly mentions AI and information architecture, suggesting genuine AI content rather than a sales pitch, and appears to be an in-person meetup event (likely Atlanta-based given the Ladies That UX ATL meetup group), but the missing location field and empty description limit confidence in the exact venue and event depth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>AI Workshop with Microsoft and Neo4j</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>4</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="n">
+        <v>46261</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>1:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/aittg-atlanta/events/316088846/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr"/>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (Microsoft and Neo4j workshop) with in-person Atlanta location, but empty description and missing venue details reduce confidence despite the clear AI focus and reputable organizers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>AI Fundamentals for Small Business Owners (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>3</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Alpharetta, GA</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-at-8-19-1</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr"/>
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>Event has clear AI content (fundamentals topic) and is in-person in Georgia (Alpharetta), but the empty description and 'small business owners' framing suggest it may be sales-oriented rather than educational, and lacks details on depth/quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>PDX AI Expo Second Webinar</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>10:00 PM</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-kul-pdx-20260820</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>Event has no AI content mentioned in title or description (only 'PDX AI Expo Second Webinar' with empty short_description), is virtual-only with no Georgia connection, and lacks sufficient details to verify any AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Batchery Startup Studio Office Hours (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>2</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-st-8-20</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr"/>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>Event mentions AI in the title ('The AI Collective') but lacks description details to confirm genuine AI content versus a generic startup office hours event, and location is blank despite in-person designation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>How To Build A One Person Company With AI</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>2</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>8:00 AM</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-kul-AIS-20260822</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr"/>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>Event title mentions AI but lacks description, location, and Georgia ties; virtual-only format with no apparent educational value or Georgia organization hosting it suggests a general webinar that may be a sales pitch rather than substantive AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Build a Second Brain for Your AI Coding Agents</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>9:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/build-a-second-brain-for-your-ai-coding-agents-registration-1997854208719?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr"/>
+      <c r="K155" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with no Georgia tie, no organization details provided, and insufficient event description to verify AI content beyond the title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>AI Tool Intensive</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>2</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-tool-intensive-tickets-1997208673907?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr"/>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>Event has clear AI focus in title but is virtual-only with no Georgia organizational tie evident, and critically lacks any description or details to verify content authenticity or distinguish it from a sales pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>FREE AI Data Engineering Bootcamp | USA Only | Join WhatsApp Group</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>2</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>10:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-ai-data-engineering-bootcamp-usa-only-join-whatsapp-group-tickets-1992777462033?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr"/>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>Event has clear AI/data engineering focus, but is virtual-only with no Georgia organizational tie, unclear host organization, and lacks substantive description details beyond the promotional title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>AI Security Intelligence Forum 1 Day in Marietta, GA</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>4</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr"/>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Marietta, GA</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-security-intelligence-forum-1-day-in-marietta-ga-tickets-1992626101309?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr"/>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>In-person event in Marietta, GA (outside metro Atlanta) with clear AI focus in title (AI Security Intelligence Forum), but incomplete event details and missing date/time information limit confidence in scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Design It, Release It — Free Live App-Building Challenge</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="n">
+        <v>46251</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/design-it-release-it-free-live-app-building-challenge-registration-1997505995203?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr"/>
+      <c r="K159" s="2" t="inlineStr">
+        <is>
+          <t>Event has no mention of AI, machine learning, or automation in its title or available description, and lacks sufficient detail to determine if any AI component exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>AI Threat Detection Summit 1 Day in Sandy Springs, GA</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>4</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Sandy Springs, GA</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-threat-detection-summit-1-day-in-sandy-springs-ga-tickets-1992637267708?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI-focused event (threat detection) in Sandy Springs, Georgia outside metro Atlanta, but lacks detailed description content to fully assess educational value versus sales pitch nature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Southeast RUG - Atlanta August 2026 - AI / ERP Education</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>4</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Oaks at Dunwoody · 1200 Abernathy Rd NE</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/southeast-rug-atlanta-august-2026-ai-erp-education-tickets-1980092625345?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr"/>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>In-person Atlanta event with explicit AI/ERP education focus, but limited detail in description and unclear whether AI is a primary or secondary component of the content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>AI Creative Launch Bootcamp at The Brio!</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>3</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Tucker · Brio Theater</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-creative-launch-bootcamp-at-the-brio-tickets-1998161340358?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr"/>
+      <c r="K162" s="2" t="inlineStr">
+        <is>
+          <t>In-person Georgia event (Tucker) with clear AI focus in title, but completely empty description prevents assessment of depth, educational value, or whether it's a genuine learning opportunity versus a sales pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Technology Health and Wealth</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>1</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Castleberry Hill · Russell Innovation Center for Entrepreneurs</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/technology-health-and-wealth-tickets-1997931976324?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or short description, triggering the automatic-1 rule, though the vague title and missing description limit confidence in this assessment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Wednesd.AI</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>4</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>North Buckhead · Atlanta Tech Village - Buckhead</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr"/>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t>In-person Atlanta AI event with clear AI focus in title, but low confidence due to missing event description that would clarify content quality and educational value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Curiosity Series #3: Why Five Stones? | Ignite House Atlanta</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>1</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>East Washington · Ignite House</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/curiosity-series-3-why-five-stones-ignite-house-atlanta-tickets-1997481419697?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr"/>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or available description, triggering the automatic-1 rule despite being in-person in Atlanta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr"/>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" s="3" t="inlineStr"/>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr"/>
+      <c r="K166" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7067,7 +8235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K215"/>
+  <dimension ref="A1:K243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -17132,7 +18300,6 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
-      <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/hacking-the-system-health-freedom-and-income-tickets-1994593661334?aff=ebdssbdestsearch</t>
@@ -17368,7 +18535,6 @@
           <t>August 10, 2026</t>
         </is>
       </c>
-      <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
           <t>Savannah, GA</t>
@@ -17509,7 +18675,6 @@
           <t>August 10, 2026</t>
         </is>
       </c>
-      <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
           <t>Augusta, GA</t>
@@ -17627,6 +18792,1314 @@
       <c r="K215" s="2" t="inlineStr">
         <is>
           <t>Event has zero mention of AI, machine learning, or automation—it is a CISSP cybersecurity certification exam prep program with no AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>TAG-Ed Pathways to Leadership Virtual Open House</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>1</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/qWFX016fkCQCe</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>Join us for an inside look at the Pathways to Leadership program, a year-long leadership experience designed for emerging and mid-level professionals. During this session, you'll learn about the program's structure and benefits and hear from graduates.</t>
+        </is>
+      </c>
+      <c r="K216" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation, and appears to be a general leadership development program open house with no AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Mid-Year Market Update presented by TAG Corporate Development Society</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>1</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/07FO6JwhxCwCR</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>The conversation will cover equity market performance, credit market functionality, M&amp;A activity, and the evolving technology investment landscape.</t>
+        </is>
+      </c>
+      <c r="K217" s="2" t="inlineStr">
+        <is>
+          <t>The event description makes no mention of AI, machine learning, or automation—it focuses on equity markets, credit markets, and M&amp;A activity with only vague reference to 'technology investment landscape' which does not constitute genuine AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Find a Startup to Help or Join</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>1</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D218" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/projects-for-developers-cs-majors-and-ux-designers/events/314898432/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr"/>
+      <c r="K218" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>AI Founders Lunch &amp; Learn</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>1</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="n">
+        <v>46252</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>4:30 AM GMT+3</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Helsinki, Finland</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-fi-8-18</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr"/>
+      <c r="K219" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Finland, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Agentic AI Knight Turku</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>1</v>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D220" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>10:00 AM GMT+3</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Turku, Finland</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-fi-8-19</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr"/>
+      <c r="K220" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Finland, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Building with AI: Stamford Micro-Hackathon (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>1</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Stamford, CT</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-st-8-19</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr"/>
+      <c r="K221" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Connecticut (CT), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Social Happy Hour (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>1</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Detroit, MI</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-de-8-19</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr"/>
+      <c r="K222" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Michigan (MI), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Prompting Desvelado: Secretos que Funcionan (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>1</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="n">
+        <v>46254</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Bogotá, Colombia</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-bog-prompt-20-8</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr"/>
+      <c r="K223" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Colombia, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Hack for Humanity: Canberra</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>1</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Acton, Australia</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>https://luma.com/h4h-canberra</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr"/>
+      <c r="K224" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Australia, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>[Beginner 101] Claude Dashboard for CEOs and HODs</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>1</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="n">
+        <v>46255</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>9:00 PM</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Puchong, Malaysia</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-kul-CMC-20260822</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr"/>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Malaysia, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Practical Agentic AI - Build with AI Series (w/ The AI Collective Pune)</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>1</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>1:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-pu-8-22</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr"/>
+      <c r="K226" s="2" t="inlineStr">
+        <is>
+          <t>Location is in India, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Build with AI &lt;/Noida&gt;</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>1</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>1:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>New Delhi, India</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-noida-build-with-ai</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr"/>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>Location is in India, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Penang Coffee Tech Talk #001</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>1</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>2:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Jelutong, Malaysia</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-kul-20260822</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr"/>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Malaysia, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Founder Brand Lab: Personal Branding Workshop for Founders (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>1</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>4:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Bengaluru, India</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-founder-personal-branding</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr"/>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>Location is in India, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>AI Security Intelligence Masterclass 1 Day in Chapel Hill, NC</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>1</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Chapel Hill, NC</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-security-intelligence-masterclass-1-day-in-chapel-hill-nc-tickets-1992624392197?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr"/>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>Location is in North Carolina (NC), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>AI Security Operations Summit 1 Day in Fremont, CA</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>1</v>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr"/>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Fremont, CA</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-security-operations-summit-1-day-in-fremont-ca-tickets-1992624395206?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr"/>
+      <c r="K231" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>AI-Powered Threat Detection 1 Day in Frisco, TX</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>1</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr"/>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Frisco, TX</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-powered-threat-detection-1-day-in-frisco-tx-tickets-1992624396209?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr"/>
+      <c r="K232" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Texas (TX), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>AI Security Analytics Training 1 Day in Katy, TX</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>1</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="inlineStr"/>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Katy, TX</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-security-analytics-training-1-day-in-katy-tx-tickets-1992626100306?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr"/>
+      <c r="K233" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Texas (TX), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>AI Threat Monitoring Summit 1 Day in Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>1</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="inlineStr"/>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr"/>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-threat-monitoring-summit-1-day-in-mountain-view-ca-tickets-1992626112342?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr"/>
+      <c r="K234" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>AI Security Operations Masterclass 1 Day in Menlo Park, CA</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>1</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="inlineStr"/>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Menlo Park, CA</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-security-operations-masterclass-1-day-in-menlo-park-ca-tickets-1992626110336?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr"/>
+      <c r="K235" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>AI Risk Analytics Workshop 1 Day in Norwalk, CT</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>1</v>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr"/>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Norwalk, CT</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-risk-analytics-workshop-1-day-in-norwalk-ct-tickets-1992626120366?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr"/>
+      <c r="K236" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Connecticut (CT), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>AI Risk Monitoring Lab 1 Day in Clearwater, FL</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>1</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr"/>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr"/>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Clearwater, FL</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-risk-monitoring-lab-1-day-in-clearwater-fl-tickets-1992624393200?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr"/>
+      <c r="K237" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Florida (FL), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>AI Security Analytics Workshop 1 Day in El Segundo, CA</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>1</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr"/>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr"/>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>El Segundo, CA</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-security-analytics-workshop-1-day-in-el-segundo-ca-tickets-1992624394203?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr"/>
+      <c r="K238" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>AI Risk Detection Workshop 1 Day in McKinney, TX</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>1</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr"/>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>McKinney, TX</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-risk-detection-workshop-1-day-in-mckinney-tx-tickets-1992626104318?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr"/>
+      <c r="K239" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Texas (TX), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>AI Security Monitoring Bootcamp 1 Day in Newark, NJ</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>1</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D240" s="3" t="inlineStr"/>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Newark, NJ</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-security-monitoring-bootcamp-1-day-in-newark-nj-tickets-1992626118360?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr"/>
+      <c r="K240" s="2" t="inlineStr">
+        <is>
+          <t>Location is in New Jersey (NJ), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Dumpling Squishy STEM Lab</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>1</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Peoplestown · 1161 Ridge Ave SW</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/dumpling-squishy-stem-lab-tickets-1996471558174?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr"/>
+      <c r="K241" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of location or in-person format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>CEH v12 Ethical Hacking Bootcamp – 4 Days Training in Savannah, GA</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>1</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>North Historic District · 100 Bull St</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ceh-v12-ethical-hacking-bootcamp-4-days-training-in-savannah-ga-tickets-1986551522079?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr"/>
+      <c r="K242" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule despite being an in-person technical security training in Georgia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Block Party South Athens</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>1</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="n">
+        <v>46256</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>August 17, 2026</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Broad Acres · Athentic Brewing Company</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/block-party-south-athens-tickets-1997878158353?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr"/>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of location or in-person status.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-08-24
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K166" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K180" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K243" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K247" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K166"/>
+  <dimension ref="A1:K180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -473,7 +473,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
@@ -7068,7 +7068,6 @@
           <t>8:30 AM - 2:00 PM</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/qWFJmQmFkCQCe</t>
@@ -7108,8 +7107,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr"/>
-      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/aimst---ai-conference---gma-special-exhibitor-and-moderator</t>
@@ -7154,7 +7151,6 @@
           <t>4:20 PM EDT</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
           <t>https://www.meetup.com/refactr-tech/events/315951068/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7199,7 +7195,6 @@
           <t>5:00 PM EDT</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316063226/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7244,7 +7239,6 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>https://www.meetup.com/freeside-atlanta/events/315371013/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7289,7 +7283,6 @@
           <t>11:45 AM EDT</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/315873146/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7383,7 +7376,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>https://www.meetup.com/blackhack-society-atlanta/events/315951497/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7428,7 +7420,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>https://www.meetup.com/ladies-that-ux-atl/events/314440739/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7473,7 +7464,6 @@
           <t>1:30 PM EDT</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
           <t>https://www.meetup.com/aittg-atlanta/events/316088846/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7616,7 +7606,6 @@
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>https://luma.com/aic-st-8-20</t>
@@ -7661,7 +7650,6 @@
           <t>8:00 AM</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>https://luma.com/aic-kul-AIS-20260822</t>
@@ -7706,7 +7694,6 @@
           <t>9:00 AM EDT</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/build-a-second-brain-for-your-ai-coding-agents-registration-1997854208719?aff=ebdssbdestsearch</t>
@@ -7751,7 +7738,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-tool-intensive-tickets-1997208673907?aff=ebdssbdestsearch</t>
@@ -7796,7 +7782,6 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-ai-data-engineering-bootcamp-usa-only-join-whatsapp-group-tickets-1992777462033?aff=ebdssbdestsearch</t>
@@ -7834,7 +7819,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>Marietta, GA</t>
@@ -7884,7 +7868,6 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/design-it-release-it-free-live-app-building-challenge-registration-1997505995203?aff=ebdssbdestsearch</t>
@@ -8202,17 +8185,12 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr"/>
-      <c r="C166" t="inlineStr"/>
       <c r="D166" s="3" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -8220,6 +8198,604 @@
       </c>
       <c r="J166" s="2" t="inlineStr"/>
       <c r="K166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Meet the Data and AI Mentor presented by TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>4</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/WqFXB5btaCJCE</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>An immersive, speed-dating style mentorship event where junior professionals connect with senior leaders in technology, data, and AI. Mentees will gain career insights, practical tips, and strategies for long-term success while building meaningful mentor-oriented relationships.</t>
+        </is>
+      </c>
+      <c r="K167" s="2" t="inlineStr">
+        <is>
+          <t>Hosted by TAG Data Science &amp; AI Society (a Georgia organization per the criteria), features AI as a core theme with senior leaders in AI/data mentoring junior professionals, and while marked virtual, the Georgia host elevates it to 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>AI in Action: Real-World Projects Transforming Fintech presented by TAG Fintech Society</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>4</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>11:30 AM - 1:30 PM</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/AnFJEbAfVCdCN</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>This Lunch &amp; Learn session will feature discussions with a series of tech and financial services leaders who have gone beyond brainstorming about how AI will impact their businesses.</t>
+        </is>
+      </c>
+      <c r="K168" s="2" t="inlineStr">
+        <is>
+          <t>TAG Fintech Society is a Georgia-based organization (TAG chapter), the event has clear AI content focused on real-world AI projects in fintech, and while the location field is blank (treated as in-person default), the virtual designation is explicit in the JSON, making this a Georgia-hosted virtual educational event on AI that scores well under the criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr"/>
+      <c r="C169" t="inlineStr"/>
+      <c r="D169" s="3" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J169" s="2" t="inlineStr"/>
+      <c r="K169" s="2" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Agentic AI Meetup - August</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>4</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>5:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/aittg-atlanta/events/315755582/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>Join us for deep dive tech talks on AI, GenAI, LLMs and Agents, hands-on experiences on code labs, workshops, and networking with speakers and fellow developers.</t>
+        </is>
+      </c>
+      <c r="K170" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (agentic AI, GenAI, LLMs, agents with tech talks and hands-on labs) hosted by Atlanta AI Tinkerers (a Georgia-based organization), in-person format, though location venue details are missing from this listing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Cybersecurity n' Chill Networking Monthly Meetup by BlackHack Society</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>4</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/blackhack-society-atlanta/events/313204276/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>Join BlackHack Society of Atlanta where young professionals and industry experts discuss the latest trends in Cybersecurity, Ethical Hacking, AI, and Offensive Security. This casual meet-and-greet over food, drinks and video games is designed for technology entrepreneurs, ethical hackers, and anyone interested in cybersecurity to connect with the local community.</t>
+        </is>
+      </c>
+      <c r="K171" s="2" t="inlineStr">
+        <is>
+          <t>In-person Atlanta event hosted by BlackHack Society with explicit mention of AI as one of several discussion topics alongside cybersecurity and ethical hacking, making it an educational networking event with genuine AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (AN OPEN AI FORUM FOR ALL)</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>2</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/315505979/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-online&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>A collaborative community where members share real experiences and help each other grow in AI. Explore topics from basic AI concepts to advanced tools, automation, prompting, business applications, and emerging technologies. Open discussion, live demos, and networking for all experience levels.</t>
+        </is>
+      </c>
+      <c r="K172" s="2" t="inlineStr">
+        <is>
+          <t>Event is virtual-only with clear AI content (AI concepts, tools, automation, prompting), but lacks Georgia-specific hosting or organizational ties, making it a national virtual event that scores below the threshold for out-of-state virtual events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Ethical Hacker Tactics, CTF &amp; Tech Talks Monthly by BlackHack Society</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>3</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/blackhack-society-atlanta/events/313204253/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>Monthly offensive security hacking practice session featuring guided practice on penetration testing techniques. Topics include Vulnhub, Google Dorking, Capture the Flag Events, Net King of the Hill, FlipperZero, Wifi Pineapple, and Locksport. Bring your laptop and Kali Linux. Guest speakers announced as scheduled.</t>
+        </is>
+      </c>
+      <c r="K173" s="2" t="inlineStr">
+        <is>
+          <t>This is an in-person security-focused event hosted by BlackHack Society in Atlanta with legitimate educational content on penetration testing and hacking techniques (which involve automation and technical security tools), but lacks explicit AI/ML mentions and is primarily about offensive security rather than AI specifically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Save millions on inference by building a model router</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>3</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-ship-and-social/events/316198820/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to route AI requests to the right models instead of sending them all to the most expensive ones. Speaker Aria will teach you why using the best model costs ~7x more than necessary, the four ways to build a router, and how to catch bad answers before users see them. You'll write your own routing rule and walk away with a working router you can read end to end in one sitting.</t>
+        </is>
+      </c>
+      <c r="K174" s="2" t="inlineStr">
+        <is>
+          <t>The event has strong AI content (model routing, inference optimization) and appears to be in-person, but the missing location prevents confirmation it's in Georgia, and the Meetup group name suggests it may be national rather than Georgia-based, though the educational technical nature of the talk is a positive factor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Agentic AI Meetup (August)</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>4</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="n">
+        <v>46258</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>5:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlantaai/events/315755600/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>Join us for deep dive tech talks on AI, GenAI, LLMs and Agents, hands-on experiences on code labs, workshops, and networking with speakers and fellow developers. In collaboration with Google.</t>
+        </is>
+      </c>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (Agentic AI, GenAI, LLMs, Agents with hands-on labs) hosted by Atlanta AI Tinkerers (a recognized Georgia organization per criteria), in-person format, educational focus with industry collaboration (Google), though the blank location field and August 2026 date prevent a perfect score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr"/>
+      <c r="C176" t="inlineStr"/>
+      <c r="D176" s="3" t="inlineStr"/>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr"/>
+      <c r="K176" s="2" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/d/united-states--georgia/science-and-tech--events--this-month/?page=1</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr"/>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" s="3" t="inlineStr"/>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 11, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 1s, resets at Mon Aug 24 2026 14:34:04 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr"/>
+      <c r="K177" s="2" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Agents, Everywhere: Beyond The Chatbot — Global Hackathon</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>5</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/p/agents-everywhere-beyond-the-chatbot-global-hackathon</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>AI Tinkerers will host a hackathon for builders to develop working agents. Sponsors OpenAI, CopilotKit, and OpenRouter will provide support.</t>
+        </is>
+      </c>
+      <c r="K178" s="2" t="inlineStr">
+        <is>
+          <t>This is a Georgia-hosted (Atlanta AI Tinkerers) in-person hackathon with explicit AI content (AI agents development), prominent AI sponsor support, and strong educational/developmental value for builders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - August</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>3</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="n">
+        <v>46260</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Manuels Tavern, 602 North Highland Ave NE, Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315044570/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>Casual BitPlebs meetup at Manuel's Tavern. Main topic: Monitoring the Situation - Red Team edition. Devs embroiled in a struggle to stay ahead of the AI and preserve freedom tech. Includes introduction, community announcements, an astrology update on AI exploits, and a beer social.</t>
+        </is>
+      </c>
+      <c r="K179" s="2" t="inlineStr">
+        <is>
+          <t>The event is hosted by ATL BitLab (a Georgia organization) in Atlanta and explicitly mentions AI as a main topic ('Red Team edition' focused on 'staying ahead of the AI'), but it's primarily a casual social meetup with beer rather than an educational or technical AI discussion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>https://ai.georgia.gov/events</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr"/>
+      <c r="C180" t="inlineStr"/>
+      <c r="D180" s="3" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 12, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 1s, resets at Mon Aug 24 2026 14:34:04 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr"/>
+      <c r="K180" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8235,7 +8811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K243"/>
+  <dimension ref="A1:K247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -18822,7 +19398,6 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/qWFX016fkCQCe</t>
@@ -18871,7 +19446,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/07FO6JwhxCwCR</t>
@@ -18920,7 +19494,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr">
         <is>
           <t>https://www.meetup.com/projects-for-developers-cs-majors-and-ux-designers/events/314898432/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -19546,7 +20119,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
           <t>Fremont, CA</t>
@@ -19589,7 +20161,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>Frisco, TX</t>
@@ -19632,7 +20203,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
           <t>Katy, TX</t>
@@ -19675,7 +20245,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
           <t>Mountain View, CA</t>
@@ -19718,7 +20287,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>Menlo Park, CA</t>
@@ -19761,7 +20329,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>Norwalk, CT</t>
@@ -19804,7 +20371,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>Clearwater, FL</t>
@@ -19847,7 +20413,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>El Segundo, CA</t>
@@ -19890,7 +20455,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>McKinney, TX</t>
@@ -19933,7 +20497,6 @@
           <t>August 17, 2026</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>Newark, NJ</t>
@@ -20100,6 +20663,198 @@
       <c r="K243" s="2" t="inlineStr">
         <is>
           <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of location or in-person status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Fiber Manufacturer Webinar presented by TAG Infrastructure Society</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>1</v>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D244" s="3" t="n">
+        <v>46266</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/4lFO3BwURCMCx</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr"/>
+      <c r="K244" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; despite being hosted by TAG (a Georgia organization), the event is about fiber manufacturing with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>TAG-Ed Pathways to Leadership Virtual Open House</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>1</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="n">
+        <v>46268</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>6:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/tag-ed-pathways-to-leadership-virtual-open-house-1848623?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>Join us for an inside look at the Pathways to Leadership program, a year-long leadership experience designed for emerging and mid-level professionals. Learn about the program's structure and benefits and hear from graduates.</t>
+        </is>
+      </c>
+      <c r="K245" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, and despite being hosted by TAG (a Georgia organization), the automatic-1 rule applies because there is no genuine AI-focused component stated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>TAG-Ed IBM SkillsBuild Orientation x Tech Women Foundation</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>1</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D246" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>6:00 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr"/>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/aZFEJ70HvCqCZ</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a mandatory virtual orientation to kick off the upcoming cohort. During this session, participants will receive an overview of the program structure, expectations, key dates, and demo on how to access the learning platform.</t>
+        </is>
+      </c>
+      <c r="K246" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it is purely an orientation for program access and logistics, triggering the automatic-1 rule despite TAG's Georgia tie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Optimized Locking in SQL Server 2025: Internals, Contention, and Concurrency</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>1</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="n">
+        <v>46273</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>August 24, 2026</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/dba-fundamentals-group/events/312863781/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-online&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr"/>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>The event contains zero mention of AI, machine learning, or automation in its title or description—it is exclusively about SQL Server locking internals, making it an automatic 1 regardless of other criteria.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert master to pre-2026-08-24 state
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K180" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K166" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K247" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K243" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K180"/>
+  <dimension ref="A1:K166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -473,7 +473,7 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
@@ -7068,6 +7068,7 @@
           <t>8:30 AM - 2:00 PM</t>
         </is>
       </c>
+      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/qWFJmQmFkCQCe</t>
@@ -7107,6 +7108,8 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/aimst---ai-conference---gma-special-exhibitor-and-moderator</t>
@@ -7151,6 +7154,7 @@
           <t>4:20 PM EDT</t>
         </is>
       </c>
+      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
           <t>https://www.meetup.com/refactr-tech/events/315951068/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7195,6 +7199,7 @@
           <t>5:00 PM EDT</t>
         </is>
       </c>
+      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316063226/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7239,6 +7244,7 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
+      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>https://www.meetup.com/freeside-atlanta/events/315371013/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7283,6 +7289,7 @@
           <t>11:45 AM EDT</t>
         </is>
       </c>
+      <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/315873146/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7376,6 +7383,7 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
+      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>https://www.meetup.com/blackhack-society-atlanta/events/315951497/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7420,6 +7428,7 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
+      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>https://www.meetup.com/ladies-that-ux-atl/events/314440739/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7464,6 +7473,7 @@
           <t>1:30 PM EDT</t>
         </is>
       </c>
+      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
           <t>https://www.meetup.com/aittg-atlanta/events/316088846/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -7606,6 +7616,7 @@
           <t>10:00 AM</t>
         </is>
       </c>
+      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>https://luma.com/aic-st-8-20</t>
@@ -7650,6 +7661,7 @@
           <t>8:00 AM</t>
         </is>
       </c>
+      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>https://luma.com/aic-kul-AIS-20260822</t>
@@ -7694,6 +7706,7 @@
           <t>9:00 AM EDT</t>
         </is>
       </c>
+      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/build-a-second-brain-for-your-ai-coding-agents-registration-1997854208719?aff=ebdssbdestsearch</t>
@@ -7738,6 +7751,7 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
+      <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-tool-intensive-tickets-1997208673907?aff=ebdssbdestsearch</t>
@@ -7782,6 +7796,7 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
+      <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-ai-data-engineering-bootcamp-usa-only-join-whatsapp-group-tickets-1992777462033?aff=ebdssbdestsearch</t>
@@ -7819,6 +7834,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>Marietta, GA</t>
@@ -7868,6 +7884,7 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
+      <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/design-it-release-it-free-live-app-building-challenge-registration-1997505995203?aff=ebdssbdestsearch</t>
@@ -8185,12 +8202,17 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr"/>
+      <c r="C166" t="inlineStr"/>
       <c r="D166" s="3" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -8198,604 +8220,6 @@
       </c>
       <c r="J166" s="2" t="inlineStr"/>
       <c r="K166" s="2" t="inlineStr"/>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>Meet the Data and AI Mentor presented by TAG Data Science &amp; AI Society</t>
-        </is>
-      </c>
-      <c r="B167" t="n">
-        <v>4</v>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D167" s="3" t="n">
-        <v>46280</v>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>5:30 PM - 7:30 PM</t>
-        </is>
-      </c>
-      <c r="G167" t="inlineStr"/>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>https://members.tagonline.org/ap/Events/Register/WqFXB5btaCJCE</t>
-        </is>
-      </c>
-      <c r="I167" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J167" s="2" t="inlineStr">
-        <is>
-          <t>An immersive, speed-dating style mentorship event where junior professionals connect with senior leaders in technology, data, and AI. Mentees will gain career insights, practical tips, and strategies for long-term success while building meaningful mentor-oriented relationships.</t>
-        </is>
-      </c>
-      <c r="K167" s="2" t="inlineStr">
-        <is>
-          <t>Hosted by TAG Data Science &amp; AI Society (a Georgia organization per the criteria), features AI as a core theme with senior leaders in AI/data mentoring junior professionals, and while marked virtual, the Georgia host elevates it to 4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>AI in Action: Real-World Projects Transforming Fintech presented by TAG Fintech Society</t>
-        </is>
-      </c>
-      <c r="B168" t="n">
-        <v>4</v>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D168" s="3" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>11:30 AM - 1:30 PM</t>
-        </is>
-      </c>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>https://members.tagonline.org/ap/Events/Register/AnFJEbAfVCdCN</t>
-        </is>
-      </c>
-      <c r="I168" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J168" s="2" t="inlineStr">
-        <is>
-          <t>This Lunch &amp; Learn session will feature discussions with a series of tech and financial services leaders who have gone beyond brainstorming about how AI will impact their businesses.</t>
-        </is>
-      </c>
-      <c r="K168" s="2" t="inlineStr">
-        <is>
-          <t>TAG Fintech Society is a Georgia-based organization (TAG chapter), the event has clear AI content focused on real-world AI projects in fintech, and while the location field is blank (treated as in-person default), the virtual designation is explicit in the JSON, making this a Georgia-hosted virtual educational event on AI that scores well under the criteria.</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>https://www.aimanufacturingconference.com/</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr"/>
-      <c r="C169" t="inlineStr"/>
-      <c r="D169" s="3" t="inlineStr"/>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr">
-        <is>
-          <t>no_events</t>
-        </is>
-      </c>
-      <c r="J169" s="2" t="inlineStr"/>
-      <c r="K169" s="2" t="inlineStr"/>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>Agentic AI Meetup - August</t>
-        </is>
-      </c>
-      <c r="B170" t="n">
-        <v>4</v>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D170" s="3" t="n">
-        <v>46258</v>
-      </c>
-      <c r="E170" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F170" t="inlineStr">
-        <is>
-          <t>5:30 PM EDT</t>
-        </is>
-      </c>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/aittg-atlanta/events/315755582/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I170" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J170" s="2" t="inlineStr">
-        <is>
-          <t>Join us for deep dive tech talks on AI, GenAI, LLMs and Agents, hands-on experiences on code labs, workshops, and networking with speakers and fellow developers.</t>
-        </is>
-      </c>
-      <c r="K170" s="2" t="inlineStr">
-        <is>
-          <t>Strong AI content (agentic AI, GenAI, LLMs, agents with tech talks and hands-on labs) hosted by Atlanta AI Tinkerers (a Georgia-based organization), in-person format, though location venue details are missing from this listing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>Cybersecurity n' Chill Networking Monthly Meetup by BlackHack Society</t>
-        </is>
-      </c>
-      <c r="B171" t="n">
-        <v>4</v>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D171" s="3" t="n">
-        <v>46280</v>
-      </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F171" t="inlineStr">
-        <is>
-          <t>6:30 PM EDT</t>
-        </is>
-      </c>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/blackhack-society-atlanta/events/313204276/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I171" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J171" s="2" t="inlineStr">
-        <is>
-          <t>Join BlackHack Society of Atlanta where young professionals and industry experts discuss the latest trends in Cybersecurity, Ethical Hacking, AI, and Offensive Security. This casual meet-and-greet over food, drinks and video games is designed for technology entrepreneurs, ethical hackers, and anyone interested in cybersecurity to connect with the local community.</t>
-        </is>
-      </c>
-      <c r="K171" s="2" t="inlineStr">
-        <is>
-          <t>In-person Atlanta event hosted by BlackHack Society with explicit mention of AI as one of several discussion topics alongside cybersecurity and ethical hacking, making it an educational networking event with genuine AI content.</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (AN OPEN AI FORUM FOR ALL)</t>
-        </is>
-      </c>
-      <c r="B172" t="n">
-        <v>2</v>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D172" s="3" t="n">
-        <v>46275</v>
-      </c>
-      <c r="E172" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>7:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/ai-growth-circle/events/315505979/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-online&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I172" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J172" s="2" t="inlineStr">
-        <is>
-          <t>A collaborative community where members share real experiences and help each other grow in AI. Explore topics from basic AI concepts to advanced tools, automation, prompting, business applications, and emerging technologies. Open discussion, live demos, and networking for all experience levels.</t>
-        </is>
-      </c>
-      <c r="K172" s="2" t="inlineStr">
-        <is>
-          <t>Event is virtual-only with clear AI content (AI concepts, tools, automation, prompting), but lacks Georgia-specific hosting or organizational ties, making it a national virtual event that scores below the threshold for out-of-state virtual events.</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>Ethical Hacker Tactics, CTF &amp; Tech Talks Monthly by BlackHack Society</t>
-        </is>
-      </c>
-      <c r="B173" t="n">
-        <v>3</v>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D173" s="3" t="n">
-        <v>46268</v>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F173" t="inlineStr">
-        <is>
-          <t>6:30 PM EDT</t>
-        </is>
-      </c>
-      <c r="G173" t="inlineStr"/>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/blackhack-society-atlanta/events/313204253/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J173" s="2" t="inlineStr">
-        <is>
-          <t>Monthly offensive security hacking practice session featuring guided practice on penetration testing techniques. Topics include Vulnhub, Google Dorking, Capture the Flag Events, Net King of the Hill, FlipperZero, Wifi Pineapple, and Locksport. Bring your laptop and Kali Linux. Guest speakers announced as scheduled.</t>
-        </is>
-      </c>
-      <c r="K173" s="2" t="inlineStr">
-        <is>
-          <t>This is an in-person security-focused event hosted by BlackHack Society in Atlanta with legitimate educational content on penetration testing and hacking techniques (which involve automation and technical security tools), but lacks explicit AI/ML mentions and is primarily about offensive security rather than AI specifically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>Save millions on inference by building a model router</t>
-        </is>
-      </c>
-      <c r="B174" t="n">
-        <v>3</v>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D174" s="3" t="n">
-        <v>46260</v>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>6:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/ai-ship-and-social/events/316198820/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J174" s="2" t="inlineStr">
-        <is>
-          <t>Learn how to route AI requests to the right models instead of sending them all to the most expensive ones. Speaker Aria will teach you why using the best model costs ~7x more than necessary, the four ways to build a router, and how to catch bad answers before users see them. You'll write your own routing rule and walk away with a working router you can read end to end in one sitting.</t>
-        </is>
-      </c>
-      <c r="K174" s="2" t="inlineStr">
-        <is>
-          <t>The event has strong AI content (model routing, inference optimization) and appears to be in-person, but the missing location prevents confirmation it's in Georgia, and the Meetup group name suggests it may be national rather than Georgia-based, though the educational technical nature of the talk is a positive factor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>Agentic AI Meetup (August)</t>
-        </is>
-      </c>
-      <c r="B175" t="n">
-        <v>4</v>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D175" s="3" t="n">
-        <v>46258</v>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>5:30 PM EDT</t>
-        </is>
-      </c>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/atlantaai/events/315755600/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J175" s="2" t="inlineStr">
-        <is>
-          <t>Join us for deep dive tech talks on AI, GenAI, LLMs and Agents, hands-on experiences on code labs, workshops, and networking with speakers and fellow developers. In collaboration with Google.</t>
-        </is>
-      </c>
-      <c r="K175" s="2" t="inlineStr">
-        <is>
-          <t>Strong AI content (Agentic AI, GenAI, LLMs, Agents with hands-on labs) hosted by Atlanta AI Tinkerers (a recognized Georgia organization per criteria), in-person format, educational focus with industry collaboration (Google), though the blank location field and August 2026 date prevent a perfect score.</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>https://luma.com/genai-collective</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr"/>
-      <c r="C176" t="inlineStr"/>
-      <c r="D176" s="3" t="inlineStr"/>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>no_events</t>
-        </is>
-      </c>
-      <c r="J176" s="2" t="inlineStr"/>
-      <c r="K176" s="2" t="inlineStr"/>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>https://www.eventbrite.com/d/united-states--georgia/science-and-tech--events--this-month/?page=1</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr"/>
-      <c r="C177" t="inlineStr"/>
-      <c r="D177" s="3" t="inlineStr"/>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr">
-        <is>
-          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 11, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 1s, resets at Mon Aug 24 2026 14:34:04 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
-        </is>
-      </c>
-      <c r="J177" s="2" t="inlineStr"/>
-      <c r="K177" s="2" t="inlineStr"/>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>Agents, Everywhere: Beyond The Chatbot — Global Hackathon</t>
-        </is>
-      </c>
-      <c r="B178" t="n">
-        <v>5</v>
-      </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D178" s="3" t="n">
-        <v>46277</v>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>10:00 AM</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr"/>
-      <c r="H178" t="inlineStr">
-        <is>
-          <t>https://atlanta.aitinkerers.org/p/agents-everywhere-beyond-the-chatbot-global-hackathon</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J178" s="2" t="inlineStr">
-        <is>
-          <t>AI Tinkerers will host a hackathon for builders to develop working agents. Sponsors OpenAI, CopilotKit, and OpenRouter will provide support.</t>
-        </is>
-      </c>
-      <c r="K178" s="2" t="inlineStr">
-        <is>
-          <t>This is a Georgia-hosted (Atlanta AI Tinkerers) in-person hackathon with explicit AI content (AI agents development), prominent AI sponsor support, and strong educational/developmental value for builders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>BitPlebs: Bitcoin Pub Night @ Manuel's Tavern - August</t>
-        </is>
-      </c>
-      <c r="B179" t="n">
-        <v>3</v>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D179" s="3" t="n">
-        <v>46260</v>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F179" t="inlineStr">
-        <is>
-          <t>6:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>Manuels Tavern, 602 North Highland Ave NE, Atlanta, GA, US</t>
-        </is>
-      </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/atlbitlab/events/315044570/?eventOrigin=group_events_list</t>
-        </is>
-      </c>
-      <c r="I179" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J179" s="2" t="inlineStr">
-        <is>
-          <t>Casual BitPlebs meetup at Manuel's Tavern. Main topic: Monitoring the Situation - Red Team edition. Devs embroiled in a struggle to stay ahead of the AI and preserve freedom tech. Includes introduction, community announcements, an astrology update on AI exploits, and a beer social.</t>
-        </is>
-      </c>
-      <c r="K179" s="2" t="inlineStr">
-        <is>
-          <t>The event is hosted by ATL BitLab (a Georgia organization) in Atlanta and explicitly mentions AI as a main topic ('Red Team edition' focused on 'staying ahead of the AI'), but it's primarily a casual social meetup with beer rather than an educational or technical AI discussion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>https://ai.georgia.gov/events</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr"/>
-      <c r="C180" t="inlineStr"/>
-      <c r="D180" s="3" t="inlineStr"/>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
-      <c r="H180" t="inlineStr"/>
-      <c r="I180" t="inlineStr">
-        <is>
-          <t>failed: Failed to scrape page with Firecrawl: Rate Limit Exceeded: Failed to scrape. Rate limit exceeded. Consumed (req/min): 12, Remaining (req/min): 0. Upgrade your plan at https://firecrawl.dev/pricing for increased rate limits or please retry after 1s, resets at Mon Aug 24 2026 14:34:04 GMT+0000 (Coordinated Universal Time) - No additional error details provided.</t>
-        </is>
-      </c>
-      <c r="J180" s="2" t="inlineStr"/>
-      <c r="K180" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8811,7 +8235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K247"/>
+  <dimension ref="A1:K243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -19398,6 +18822,7 @@
           <t>6:00 PM - 7:00 PM</t>
         </is>
       </c>
+      <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/qWFX016fkCQCe</t>
@@ -19446,6 +18871,7 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
+      <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/07FO6JwhxCwCR</t>
@@ -19494,6 +18920,7 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
+      <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr">
         <is>
           <t>https://www.meetup.com/projects-for-developers-cs-majors-and-ux-designers/events/314898432/?recId=1b4155d4-5c2a-4e60-a0af-4a1c0ccc4b94&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=cfb680a7-12bd-4219-ac05-bff87c35a5f4&amp;eventOrigin=find_page%24all</t>
@@ -20119,6 +19546,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
           <t>Fremont, CA</t>
@@ -20161,6 +19589,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>Frisco, TX</t>
@@ -20203,6 +19632,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
           <t>Katy, TX</t>
@@ -20245,6 +19675,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
           <t>Mountain View, CA</t>
@@ -20287,6 +19718,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>Menlo Park, CA</t>
@@ -20329,6 +19761,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>Norwalk, CT</t>
@@ -20371,6 +19804,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>Clearwater, FL</t>
@@ -20413,6 +19847,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>El Segundo, CA</t>
@@ -20455,6 +19890,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>McKinney, TX</t>
@@ -20497,6 +19933,7 @@
           <t>August 17, 2026</t>
         </is>
       </c>
+      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>Newark, NJ</t>
@@ -20663,198 +20100,6 @@
       <c r="K243" s="2" t="inlineStr">
         <is>
           <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating regardless of location or in-person status.</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="inlineStr">
-        <is>
-          <t>Fiber Manufacturer Webinar presented by TAG Infrastructure Society</t>
-        </is>
-      </c>
-      <c r="B244" t="n">
-        <v>1</v>
-      </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D244" s="3" t="n">
-        <v>46266</v>
-      </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F244" t="inlineStr">
-        <is>
-          <t>12:00 PM - 1:00 PM</t>
-        </is>
-      </c>
-      <c r="G244" t="inlineStr"/>
-      <c r="H244" t="inlineStr">
-        <is>
-          <t>https://members.tagonline.org/ap/Events/Register/4lFO3BwURCMCx</t>
-        </is>
-      </c>
-      <c r="I244" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J244" s="2" t="inlineStr"/>
-      <c r="K244" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; despite being hosted by TAG (a Georgia organization), the event is about fiber manufacturing with no stated AI component.</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="inlineStr">
-        <is>
-          <t>TAG-Ed Pathways to Leadership Virtual Open House</t>
-        </is>
-      </c>
-      <c r="B245" t="n">
-        <v>1</v>
-      </c>
-      <c r="C245" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D245" s="3" t="n">
-        <v>46268</v>
-      </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F245" t="inlineStr">
-        <is>
-          <t>6:00 PM - 7:00 PM</t>
-        </is>
-      </c>
-      <c r="G245" t="inlineStr"/>
-      <c r="H245" t="inlineStr">
-        <is>
-          <t>https://members.tagonline.org/calendar/Details/tag-ed-pathways-to-leadership-virtual-open-house-1848623?sourceTypeId=Website</t>
-        </is>
-      </c>
-      <c r="I245" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J245" s="2" t="inlineStr">
-        <is>
-          <t>Join us for an inside look at the Pathways to Leadership program, a year-long leadership experience designed for emerging and mid-level professionals. Learn about the program's structure and benefits and hear from graduates.</t>
-        </is>
-      </c>
-      <c r="K245" s="2" t="inlineStr">
-        <is>
-          <t>The event has zero mention of AI, machine learning, or automation in its title or description, and despite being hosted by TAG (a Georgia organization), the automatic-1 rule applies because there is no genuine AI-focused component stated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="inlineStr">
-        <is>
-          <t>TAG-Ed IBM SkillsBuild Orientation x Tech Women Foundation</t>
-        </is>
-      </c>
-      <c r="B246" t="n">
-        <v>1</v>
-      </c>
-      <c r="C246" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D246" s="3" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F246" t="inlineStr">
-        <is>
-          <t>6:00 PM - 8:00 PM</t>
-        </is>
-      </c>
-      <c r="G246" t="inlineStr"/>
-      <c r="H246" t="inlineStr">
-        <is>
-          <t>https://members.tagonline.org/ap/Events/Register/aZFEJ70HvCqCZ</t>
-        </is>
-      </c>
-      <c r="I246" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J246" s="2" t="inlineStr">
-        <is>
-          <t>Join us for a mandatory virtual orientation to kick off the upcoming cohort. During this session, participants will receive an overview of the program structure, expectations, key dates, and demo on how to access the learning platform.</t>
-        </is>
-      </c>
-      <c r="K246" s="2" t="inlineStr">
-        <is>
-          <t>The event description contains zero mention of AI, machine learning, or automation—it is purely an orientation for program access and logistics, triggering the automatic-1 rule despite TAG's Georgia tie.</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="inlineStr">
-        <is>
-          <t>Optimized Locking in SQL Server 2025: Internals, Contention, and Concurrency</t>
-        </is>
-      </c>
-      <c r="B247" t="n">
-        <v>1</v>
-      </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D247" s="3" t="n">
-        <v>46273</v>
-      </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>August 24, 2026</t>
-        </is>
-      </c>
-      <c r="F247" t="inlineStr">
-        <is>
-          <t>12:00 PM EDT</t>
-        </is>
-      </c>
-      <c r="G247" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="H247" t="inlineStr">
-        <is>
-          <t>https://www.meetup.com/dba-fundamentals-group/events/312863781/?recId=09697859-f96d-4fab-a35e-1add97ec4ec7&amp;recSource=ml-popular-events-nearby-online&amp;searchId=cbfb4fa0-571c-4ddf-bff3-26a32f00c328&amp;eventOrigin=find_page%24all</t>
-        </is>
-      </c>
-      <c r="I247" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="J247" s="2" t="inlineStr"/>
-      <c r="K247" s="2" t="inlineStr">
-        <is>
-          <t>The event contains zero mention of AI, machine learning, or automation in its title or description—it is exclusively about SQL Server locking internals, making it an automatic 1 regardless of other criteria.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-08-31
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K180" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K189" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K258" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K264" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K180"/>
+  <dimension ref="A1:K189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8226,7 +8226,6 @@
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr"/>
       <c r="H167" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/WqFXB5btaCJCE</t>
@@ -8275,7 +8274,6 @@
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr"/>
       <c r="H168" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/AnFJEbAfVCdCN</t>
@@ -8303,17 +8301,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr"/>
-      <c r="C169" t="inlineStr"/>
       <c r="D169" s="3" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
           <t>August 24, 2026</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -8349,7 +8342,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr"/>
       <c r="H170" t="inlineStr">
         <is>
           <t>https://www.meetup.com/blackhack-society-atlanta/events/313204276/?recId=87223c12-7c50-4a2a-b9d4-cb14dd08262e&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=77bf5e21-1b7b-4bbf-b4a1-a60c6109ecc9&amp;eventOrigin=find_page%24all</t>
@@ -8398,7 +8390,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr"/>
       <c r="H171" t="inlineStr">
         <is>
           <t>https://www.meetup.com/blackhack-society-atlanta/events/313204253/?recId=87223c12-7c50-4a2a-b9d4-cb14dd08262e&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=77bf5e21-1b7b-4bbf-b4a1-a60c6109ecc9&amp;eventOrigin=find_page%24all</t>
@@ -8447,7 +8438,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr">
         <is>
           <t>https://www.meetup.com/ai-ship-and-social/events/316198820/?recId=87223c12-7c50-4a2a-b9d4-cb14dd08262e&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=77bf5e21-1b7b-4bbf-b4a1-a60c6109ecc9&amp;eventOrigin=find_page%24all</t>
@@ -8496,7 +8486,6 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr"/>
       <c r="H173" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atl-ai/events/314482312/?recId=87223c12-7c50-4a2a-b9d4-cb14dd08262e&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=77bf5e21-1b7b-4bbf-b4a1-a60c6109ecc9&amp;eventOrigin=find_page%24all</t>
@@ -8524,17 +8513,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr"/>
-      <c r="C174" t="inlineStr"/>
       <c r="D174" s="3" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
           <t>August 24, 2026</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -8676,7 +8660,6 @@
           <t>6:00 PM CDT</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-studio-builder-lab-build-your-first-ai-powered-website-tickets-1998389681332?aff=ebdssbdestsearch</t>
@@ -8725,7 +8708,6 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-training-for-business-owners-get-out-of-the-day-to-day-free-live-tickets-1997983763220?aff=ebdssbdestsearch</t>
@@ -8774,7 +8756,6 @@
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
           <t>https://atlanta.aitinkerers.org/p/agents-everywhere-beyond-the-chatbot-global-hackathon</t>
@@ -8802,17 +8783,12 @@
           <t>https://www.meetup.com/atlbitlab/events/</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr"/>
-      <c r="C180" t="inlineStr"/>
       <c r="D180" s="3" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
           <t>August 24, 2026</t>
         </is>
       </c>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
-      <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -8820,6 +8796,415 @@
       </c>
       <c r="J180" s="2" t="inlineStr"/>
       <c r="K180" s="2" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Techlanta 2026</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>4</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Georgia Tech's Historic Academy of Medicine</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/techlanta-2026</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>Don't miss this opportunity to connect with Atlanta's innovation ecosystem and help shape the future of AI, XR, robotics, advanced manufacturing, and emerging technology adoption.</t>
+        </is>
+      </c>
+      <c r="K181" s="2" t="inlineStr">
+        <is>
+          <t>In-person event at Georgia Tech with explicit AI focus as a stated theme alongside other emerging technologies, though the description lacks specific session or speaker details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>TAG Data Science &amp; AI Summit 2026: Building the AI-Powered Enterprise presented by TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>5</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="n">
+        <v>46343</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>8:00 AM - 4:30 PM</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/OOFvaqjSaCqCD</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>The TAG Data Science &amp; AI Summit 2026 is a full-day Atlanta experience connecting executive strategy with applied implementation.</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>This is a full-day, in-person AI conference hosted by TAG Data Science &amp; AI Society (a Georgia organization) in Atlanta with clear AI focus on enterprise implementation, meeting all top-tier criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr"/>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" s="3" t="inlineStr"/>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr"/>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr"/>
+      <c r="K183" s="2" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Give AI the Repeat Work, Not the Keys: Build an AI Ops Layer Safely</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>2</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-for-agencies/events/316271485/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-online&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to build a secure AI operations layer that connects your tools, workflows, and data through controlled access and human guardrails. Discover how to automate audits, reporting, QA, and repeatable processes while keeping humans in control of what impacts customers and revenue.</t>
+        </is>
+      </c>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>Event is virtual-only with clear AI content but lacks Georgia organizational affiliation or Georgia-specific focus, making it a national webinar that scores at the virtual-only floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>GA AI Alliance Networking Lunch</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>4</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>11:45 AM EDT</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316283308/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>Informal networking lunch for AI professionals across Georgia. Connect with others in the AI community, share what you're working on, and build relationships. Whether you're building with AI, driving adoption, or staying current with developments, join this open invitation event.</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>Georgia-based AI community event (GA AI Alliance) with clear AI focus, in-person networking format, and statewide Georgia audience, though it's a social networking event rather than educational content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr"/>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" s="3" t="inlineStr"/>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr"/>
+      <c r="K186" s="2" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Agents, Everywhere: Bots, Channels, &amp; More — Global Hackathon</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>5</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/p/agents-everywhere-bots-channels-more-global-hackathon</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>AI Tinkerers will host a hackathon challenging builders to integrate agents into various environments. Sponsors like OpenAI will provide resources for this in-person event.</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (agents, bots, hackathon challenge), hosted by Atlanta AI Tinkerers (Georgia organization), in-person event with clear technical focus and industry backing from OpenAI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Snowday 2026: Accelerating Georgia's Data-Driven Future</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>5</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>8:30 a.m.</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>https://ai.georgia.gov/events/2026-10-20/snowday-2026</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>A one-day event bringing together Georgia state and Atlanta city leaders to share best practices in data modernization, analytics, AI and digital service transformation. Features customer stories, panel discussions, live demonstrations in public safety, health services, transportation and higher education, hands-on labs, and networking opportunities.</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>Excellent fit: in-person event in Atlanta with explicit AI content (AI and data modernization as stated themes), hosted by Georgia state government, featuring panels, demonstrations, and labs across multiple sectors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026 Georgia Emerging Technology Summit: Data &amp; AI</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>5</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="n">
+        <v>46338</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>8:00 a.m.</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>https://ai.georgia.gov/events/2026-11-12/2026-emerging-tech-summit</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr"/>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>Multi-day AI/data conference hosted by Georgia's official AI office in Atlanta with clear AI focus in the title, meeting all criteria for excellent fit.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8835,7 +9220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K258"/>
+  <dimension ref="A1:K264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -20717,7 +21102,6 @@
           <t>12:00 PM</t>
         </is>
       </c>
-      <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/4lFO3BwURCMCx</t>
@@ -20762,7 +21146,6 @@
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/tag-ed-pathways-to-leadership-virtual-open-house-1848623?sourceTypeId=Website</t>
@@ -20811,7 +21194,6 @@
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/aZFEJ70HvCqCZ</t>
@@ -20909,7 +21291,6 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
-      <c r="G248" t="inlineStr"/>
       <c r="H248" t="inlineStr">
         <is>
           <t>https://www.meetup.com/freeside-atlanta/events/315518448/?recId=87223c12-7c50-4a2a-b9d4-cb14dd08262e&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=77bf5e21-1b7b-4bbf-b4a1-a60c6109ecc9&amp;eventOrigin=find_page%24all</t>
@@ -21007,7 +21388,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G250" t="inlineStr"/>
       <c r="H250" t="inlineStr">
         <is>
           <t>https://www.meetup.com/projects-for-developers-cs-majors-and-ux-designers/events/315518454/?recId=87223c12-7c50-4a2a-b9d4-cb14dd08262e&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=77bf5e21-1b7b-4bbf-b4a1-a60c6109ecc9&amp;eventOrigin=find_page%24all</t>
@@ -21052,7 +21432,6 @@
           <t>5:00 PM CDT</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1998674450083?aff=ebdssbdestsearch</t>
@@ -21188,7 +21567,6 @@
           <t>August 24, 2026</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>Macon, GA</t>
@@ -21340,7 +21718,6 @@
           <t>3:00 PM CDT</t>
         </is>
       </c>
-      <c r="G257" t="inlineStr"/>
       <c r="H257" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/tech-and-wealth-workshop-tickets-1998759249721?aff=ebdssbdestsearch</t>
@@ -21385,7 +21762,6 @@
           <t>8:00 AM EDT</t>
         </is>
       </c>
-      <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-cybersecurity-bootcamp-usa-only-live-online-tickets-1996169284064?aff=ebdssbdestsearch</t>
@@ -21400,6 +21776,308 @@
       <c r="K258" s="2" t="inlineStr">
         <is>
           <t>Event is virtual-only with no Georgia host tie and no AI/machine learning/automation content in title or description, only cybersecurity bootcamp training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Georgia Rural Health Transformation presented by TAG Digital Health Society</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>1</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/georgia-rural-health-transformation-presented-by-tag-digital-health-society-1910658?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>A discussion exploring the impact of new approaches to workforce development, digital health, care delivery, rural hospital sustainability, maternal health, and community-based partnerships to strengthen Georgia's rural healthcare system amid workforce shortages, limited access to care, and infrastructure gaps.</t>
+        </is>
+      </c>
+      <c r="K259" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation despite being hosted by TAG Digital Health Society, and discusses only rural healthcare policy, workforce development, and care delivery with no stated AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Out of Office Hours (Social)</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>1</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr"/>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/315893352/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>A casual happy hour to connect with others across the Atlanta tech community in a relaxed, social setting. Meet new people, catch up with familiar faces, and expand your network. Food and drinks available for purchase.</t>
+        </is>
+      </c>
+      <c r="K260" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is purely a social happy hour with no AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Bytes &amp; Bites @ Krog St Market</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>1</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>11:45 AM EDT</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Krog St Market</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/315803181/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>A casual, community-driven lunch where technologists of all backgrounds come together to connect, swap ideas, and build relationships over good food. Easy, low-pressure networking with no agenda—just lunch and conversation.</t>
+        </is>
+      </c>
+      <c r="K261" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is purely a casual networking lunch with no stated AI-focused component, panel, speaker, or theme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Python Atlanta Meetup (In Person!)</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>1</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>7:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr"/>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/python-atlanta/events/315306147/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>A social gathering for the Atlanta Python Programmers community to discuss topics with formal talks scheduled. The meeting starts at 7:30PM, with optional dinner and socializing from 6:00-7:30PM beforehand.</t>
+        </is>
+      </c>
+      <c r="K262" s="2" t="inlineStr">
+        <is>
+          <t>The event description makes no mention of AI, machine learning, or automation—it is a general Python programming meetup with no stated AI-focused component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Open House!</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>1</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>7:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/freeside-atlanta/events/316117768/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>A quick meeting to introduce everyone and update on projects and equipment, followed by an informal open house where people can chat, take a tour, and check out the space. Freeside Atlanta is a 501(c)(3) non-profit for engineers, programmers, inventors, artists, and collaborators.</t>
+        </is>
+      </c>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation - it is a general open house for a makerspace with no stated AI-focused component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Nostr Atlanta #17 - Rush Hour Avoidance</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>1</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D264" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>August 31, 2026</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>4:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>684 John Wesley Dobbs Ave NE suite a1, Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/316328827/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>Join us for Nostr Atlanta! Trying to avoid the nasty rush hour traffic. Bring your laptop as this session will involve some tool building. Informal round-table discussion of Nostr and adjacent topics from 4:30–6:00 PM.</t>
+        </is>
+      </c>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a Nostr (a decentralized social protocol) meetup with tool building and discussion, which falls outside the AI criteria despite being hosted by ATL BitLab, a Georgia organization.</t>
         </is>
       </c>
     </row>

</xml_diff>